<commit_message>
gk-008: add reference field with em dash placeholder
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z15"/>
+  <dimension ref="A1:Z16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:21</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
+          <t>2026-07-05T19:34:22</t>
         </is>
       </c>
     </row>
@@ -2084,9 +2084,6 @@
           <t>良泉藏泉</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr">
         <is>
           <t>images/DE-002.jpg</t>
@@ -2102,11 +2099,125 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-05T19:10:14</t>
-        </is>
-      </c>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
+          <t>2026-07-05T19:34:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GK-008</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MACEDONIA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>马其顿·亚历山大三世 大帝 四德拉克马</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MACEDONIA · ALEXANDER III</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>BC 336-323</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Tetradrachm 四德拉克马</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Silver 银 · 26mm · 16.9g</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Price 2168; HGC 3, 1077</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>greek</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>正面: 赫拉克勒斯狮皮盔头像</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>背面: 宙斯持鹰坐像 · ΑΛΕΞΑΝΔΡΟΥ（亚历山大的）</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>亚历山大, 希腊化, 四德, 马其顿, 赫拉克勒斯, 宙斯</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>¥4,000</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>4000</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>达爷</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>私洽</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>images/GK-008.jpg</t>
+        </is>
+      </c>
+      <c r="V16" t="n">
+        <v>484405</v>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>亚历山大三世（大帝，356-323 BC）统一希腊、征服波斯，建立了人类历史上第一个横跨欧亚非的超级帝国。他对货币体系的改革影响深远：四德拉克马银币以赫拉克勒斯头像为正面，宙斯持鹰坐像为背面，成为帝国扩张的战略工具与文化符号。随着亚历山大的征服，这套币制被推广至从埃及到印度河的广大地区，继业者纷纷仿铸。利西普斯（ Lysippos ）风格的赫拉克勒斯肖像极具古典理想美，而宙斯坐像手持雄鹰的形象则强化了王权的神圣性。此枚米勒都斯（Miletus）铸币约 BC 325-320 年所见宙斯底座无碑铭，为亚历山大在世时期的早期铸型。</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>2026-07-05T19:34:22</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
version 2026070520 snapshot: 16 cards complete (GR-001, ROM-001~004, GK-002~009, UK-001, DE-001~002)
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z16"/>
+  <dimension ref="A1:Z17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:21</t>
+          <t>2026-07-05T20:14:11</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
+          <t>2026-07-05T20:14:12</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Price 2168; HGC 3, 1077</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2192,7 +2192,6 @@
           <t>私洽</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2204,7 +2203,7 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>484405</v>
+        <v>484438</v>
       </c>
       <c r="W16" t="inlineStr">
         <is>
@@ -2213,11 +2212,123 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-05T19:34:22</t>
-        </is>
-      </c>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
+          <t>2026-07-05T20:14:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GK-009</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ATHENS</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>雅典城·新式猫头鹰 四德拉克马</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ATHENS · NEW STYLE OWL</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>BC 2nd-1st Century</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Tetradrachm 四德拉克马</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Silver 银 · 31.6mm · 16.7g</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>greek</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>正面: 雅典娜女神戴阿提卡式头盔头像</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>背面: 猫头鹰立于双耳陶罐上 · 橄榄枝环绕 · ΑΘΕ</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>雅典, 猫头鹰, 希腊化, 四德, 雅典娜</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>¥13,500</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>13500</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>大象古币</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>私洽</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>images/GK-009.jpg</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>雅典猫头鹰银币是古希腊最具代表性的货币，从公元前5世纪延续至公元前1世纪，成为古代地中海世界的硬通货。古典时期结束后，雅典于公元前2世纪摆脱马其顿控制，重启银币铸造，采用全新设计风格——新式猫头鹰（New Style）。与古典版相比，新式猫头鹰正面雅典娜头像更为精致，头戴装饰丰富的阿提卡式头盔；背面猫头鹰立于双耳陶罐（amphora）之上，周边环绕橄榄枝，并刻有地方官姓名与徽记，体现了希腊化时期雅典城邦的自治与繁荣。</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>2026-07-05T20:14:12</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
GK-010: replace dual images with composite photo
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:Z18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:11</t>
+          <t>2026-07-06T16:15:38</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:38</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:38</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:38</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:38</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:38</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:38</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:39</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:39</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:39</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:39</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:39</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:39</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:39</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
+          <t>2026-07-06T16:15:39</t>
         </is>
       </c>
     </row>
@@ -2254,7 +2254,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2305,7 +2305,6 @@
           <t>私洽</t>
         </is>
       </c>
-      <c r="S17" t="inlineStr"/>
       <c r="T17" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2316,7 +2315,9 @@
           <t>images/GK-009.jpg</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr"/>
+      <c r="V17" t="n">
+        <v>973582</v>
+      </c>
       <c r="W17" t="inlineStr">
         <is>
           <t>雅典猫头鹰银币是古希腊最具代表性的货币，从公元前5世纪延续至公元前1世纪，成为古代地中海世界的硬通货。古典时期结束后，雅典于公元前2世纪摆脱马其顿控制，重启银币铸造，采用全新设计风格——新式猫头鹰（New Style）。与古典版相比，新式猫头鹰正面雅典娜头像更为精致，头戴装饰丰富的阿提卡式头盔；背面猫头鹰立于双耳陶罐（amphora）之上，周边环绕橄榄枝，并刻有地方官姓名与徽记，体现了希腊化时期雅典城邦的自治与繁荣。</t>
@@ -2324,11 +2325,125 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-05T20:14:12</t>
-        </is>
-      </c>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
+          <t>2026-07-06T16:15:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GK-010</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>LAODIKEIA AD LYCUM</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>弗里几亚劳迪西亚城·蛇篮式四德拉克马</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>LAODIKEIA AD LYCUM · SERPENT FROM CISTA MYSTICA</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>公元前133-前67年</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Tetradrachm 四德拉克马</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Silver 银 · 27.5mm · 12.56g</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>greek</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>正面: 蛇正从篮中爬出，周围常春藤花环环绕，花叶饱满</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>背面: 两条蛇缠绕弓箭袋 · AΠOΛΛΩNIOΣ ΕΥΑΡΧΟΥ · 左下角ΛΑΟ</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>蛇篮, 劳迪西亚, 弗里几亚, 罗马统治, 狄奥尼索斯, 常春藤</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>¥2,888</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>2888</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>熊太乐</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>私洽</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>images/GK-010.jpg</t>
+        </is>
+      </c>
+      <c r="V18" t="n">
+        <v>810259</v>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>蛇篮（Cista Mystica）是古希腊祭祀酒神狄奥尼索斯仪式中的神圣器物——一个装有幼蛇的柳编篮子，祭司将其取出让蛇爬出，以此象征神迹与重生。这一意象被广泛铸造在银币背面，成为古希腊钱币中最具神秘感的经典图式。此币正面蛇从篮中爬出，周围常春藤花环环绕；背面双蛇缠绕弓箭袋，铭文「AΠOΛΛΩNIOΣ ΕΥΑΡΧΟΥ」清晰漂亮——地方行政官阿波罗尼奥斯，尤阿尔科斯之子。公元前133年帕加马王国灭亡，小亚细亚落入罗马人之手，此币恐由罗马总督发行，兑换比率为三枚狄纳里银币换一枚蛇篮四德拉克马。</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>2026-07-06T16:15:39</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add GK-012: Seleucus I Nicator Bronze Chalkous, Elephant & Bucephalus, Apamaea on the Orontes
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z18"/>
+  <dimension ref="A1:Z20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:38</t>
+          <t>2026-07-06T16:54:57</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:38</t>
+          <t>2026-07-06T16:54:57</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:38</t>
+          <t>2026-07-06T16:54:57</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:38</t>
+          <t>2026-07-06T16:54:57</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:38</t>
+          <t>2026-07-06T16:54:57</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:38</t>
+          <t>2026-07-06T16:54:57</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:38</t>
+          <t>2026-07-06T16:54:57</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:39</t>
+          <t>2026-07-06T16:54:57</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:39</t>
+          <t>2026-07-06T16:54:57</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:39</t>
+          <t>2026-07-06T16:54:58</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:39</t>
+          <t>2026-07-06T16:54:58</t>
         </is>
       </c>
     </row>
@@ -1807,12 +1807,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>维多利亚 禧年头像克朗银币</t>
+          <t>维多利亚·马剑·克朗银币</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>UNITED KINGDOM · Victoria Jubilee Head · 1887</t>
+          <t>UNITED KINGDOM · Victoria · St. George &amp; Dragon · 1887</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>背面: [待补充]</t>
+          <t>背面: 圣乔治策马刺剑，斗篷飞扬，长矛刺杀毒龙，骏马前蹄腾空；龙蜷于马蹄下，翅膀伸展；底部 exergue 内镌 1887；Pistrucci 经典马剑图</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:39</t>
+          <t>2026-07-06T16:54:58</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:39</t>
+          <t>2026-07-06T16:54:58</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:39</t>
+          <t>2026-07-06T16:54:58</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:39</t>
+          <t>2026-07-06T16:54:58</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:39</t>
+          <t>2026-07-06T16:54:58</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2418,6 @@
           <t>私洽</t>
         </is>
       </c>
-      <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2430,7 +2429,7 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>810259</v>
+        <v>3871047</v>
       </c>
       <c r="W18" t="inlineStr">
         <is>
@@ -2439,11 +2438,238 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-06T16:15:39</t>
-        </is>
-      </c>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
+          <t>2026-07-06T16:54:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>GK-011</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>CYRENE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>昔兰尼阿波罗-忘忧草2德拉克马</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CYRENE · APOLLO CARNEIUS &amp; SILPHIUM</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>公元前294-前275年</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Didrachm 2德拉克马</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Silver 银 · 19mm · 7.62g</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>greek</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>正面: 阿波罗·卡内奥斯（Apollo Carneius）侧面头像 · 年轻俊美 · 羊角与桂冠共存</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>背面: Silphium忘忧草 · 茎粗壮 · 心形果实 · 卷曲根系</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>昔兰尼, 阿波罗, 忘忧草, Silphium, 塞琉古, 罗马统治, 避孕, 灭绝植物</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>¥5,500</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>5500</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>熊太乐</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>私洽</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>images/GK-011.jpg</t>
+        </is>
+      </c>
+      <c r="V19" t="n">
+        <v>3492219</v>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>昔兰尼（Cyrenaica，今利比亚东部）于公元前631年建城，相传由一群来自帖飞的移民在阿波罗神谕指引下建立。此城迅速崛起为古代世界最富庶的城邦之一，全赖一种神奇植物——Silphium（又名忘忧草， Laserpitium silphium）。这种形似巨大茴香的伞形科植物，只生长在昔兰尼周边海岸，拥有令人惊叹的医疗功效，尤其以高效的避孕作用闻名——古代妇女将其汁液涂抹于子宫口，成功率接近百分之百。其贸易价值极高，一磅Silphium的价格相当于一个罗马士兵六年的薪俸，罗马元老院甚至在其铸造的银币上压制Silphium图案，作为帝国繁荣的象征。塞琉古帝国在公元前3世纪初攻占昔兰尼后废止本地铸币，此币发行于城市沦陷后的罗马统治早期，由当地官员以原塞琉古模具或本地模具发行，正面阿波罗·卡内奥斯（Apollo Carneius，羊角神）头像，羊角与桂冠共存，象征城邦保护神的神圣权威；背面Silphium枝叶繁茂，茎粗壮有力，果实心脏形，根系卷曲——这一经典图式在昔兰尼钱币上延续了两百余年。令人唏嘘的是，公元1世纪Silphium已彻底灭绝，原因可能是过度采集、地震破坏与土壤退化三重打击。</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>2026-07-06T16:54:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GK-012</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SELEUCID EMPIRE</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>塞琉古帝国塞琉古一世铜币</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>SELEUCID EMPIRE · ELEPHANT &amp; BUCERAS</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>公元前312-前281年</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Chalkous 铜币</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Bronze 青铜 · 22mm · 6.42g</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>greek</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>正面: 亚洲象向右行走 · 体态健壮 · 背上驮有辎重</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>背面: 戴牛角之马头向右 · 下方船锚 ⚓ · 铭文 ΒΑΣΙΛΕΩΣ ΣΕΛΕΥΚΟΥ</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>塞琉古, 塞琉古一世, 胜利者, Nikator, 亚洲象, 布克法罗斯, Bucephalus, 阿帕美亚, 伊普苏斯, 继业者战争, 船锚</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>¥360</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>360</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>西西里晚祷</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>私洽</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>images/GK-012.jpg</t>
+        </is>
+      </c>
+      <c r="V20" t="n">
+        <v>175619</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>公元前323年亚历山大大帝骤然离世，其帝国随即陷入继业者战争（War of the Diadochi）。塞琉古（Seleucus）作为亚历山大的近身护卫官，于公元前321年被迫流亡埃及。公元前312年，在托勒密一世的支持下，塞琉古重返巴比伦，宣布独立，开启了塞琉古帝国长达两百余年的统治，是年便成为塞琉古纪元的元年。公元前301年伊普苏斯战役（Battle of Ipsus），塞琉古与利西马科斯（Lysimachus）联手击败安提柯（Antigonus），瓜分亚历山大帝国的东部版图，塞琉古一跃成为从安纳托利亚延伸至印度的庞大帝国之君，领土面积仅次于孔雀王朝印度。 阿帕美亚（Apamaea on the Orontes）位于奥隆特斯河畔，是塞琉古帝国最繁华的城市之一，以其母——塞琉古一世之妻阿帕美亚（Apama）命名，与安条克、塞琉西亚并列为帝国三大都城。 此币正面亚洲象向右行走，象征塞琉古从印度孔雀王朝君主旃陀罗笈多（Chandragupta）手中换取的五百头战象，这些战象是伊普苏斯战役决定性胜利的关键；背面戴牛角之马头为布克法罗斯（Bucephalus）的形象，据传是亚历山大大帝的传奇坐骑，塞琉古以布克法罗斯自比，昭示其作为亚历山大正统继承人的身份；船锚则暗指塞琉古大腿根部形似锚状的胎记，同时也象征其祖先尼卡托尔（Nicator，意为「胜利者」）作为亚历山大海军指挥官与腓力二世时期的海军将领之出身，将希腊世界的海上传统与新帝国紧紧相连。</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>2026-07-06T16:54:58</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add ROM-005: 君士坦丁一世追思币 (Divus Constantinus I Memorial Issue, AD 337-340)
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z20"/>
+  <dimension ref="A1:Z21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:57</t>
+          <t>2026-07-06T17:05:30</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:57</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:57</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:57</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:57</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:57</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:57</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:57</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:57</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:58</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:58</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:58</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:58</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:58</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:58</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:58</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:58</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:58</t>
+          <t>2026-07-06T17:05:31</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2644,6 @@
           <t>私洽</t>
         </is>
       </c>
-      <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2665,11 +2664,125 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-06T16:54:58</t>
-        </is>
-      </c>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
+          <t>2026-07-06T17:05:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ROM-005</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>DIVVS CONSTANTINVS PT AVGG</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>君士坦丁一世追思币</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>DIVVS CONSTANTINVS PT AVGG · VENERANDA MEMORIA</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>AD 337-340</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>AE2 / Nummus 青铜币</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Bronze 青铜 · 16mm · 2.18g</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>VF</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>roman</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>正面: 戴维露姆面纱的君士坦丁一世半身像向右 · 铭文 DV CONSTANTINVS PT AVGG（神化君主君士坦丁，诸帝之父）</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>背面: 君士坦丁穿托加盖头之站姿全身像 · 铭文 VN - MR（Veneranda Memoria 应受崇敬之记忆）· 底注 CONST（君士坦丁堡造币厂）</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>罗马帝国, 君士坦丁一世, Divus, 追思币, 封神, Consecratio, 君士坦提乌斯二世, VN-MR, Veneranda Memoria, 君士坦丁堡, 4世纪, 晚期罗马, 三兄共治</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>¥100</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>西西里晚祷</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>私洽</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>images/ROM-005.jpg</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>163390</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>公元337年5月22日，君士坦丁大帝（Constantinus I，公元306-337年在位）在尼科米底亚驾崩，结束了对罗马帝国近三十年的统治。这位在位期间颁布《米兰敕令》（313年）、召开尼西亚公会议（325年）、迁都博斯普鲁斯海峡并以「新罗马」命名新都的皇帝，是罗马世界最具变革意义的统治者之一。 君士坦丁驾崩后，其三位子嗣——君士坦丁二世、君士坦提乌斯二世、君士坦斯——共同继承帝位，史称「三兄共治」（337-340年）。按照罗马传统，前任皇帝在驾崩后即被元老院封神（Consecratio），纳入罗马神祇之列并享有祭祀。新任诸帝随即在各大造币厂发行追思币（Memorial Issue / Divus Issue），纪念亡父之「成神」，并以铭文宣告其「诸帝之父」（Pater Augustorum）的崇高地位。 此枚追思币为君士坦提乌斯二世（Constantius II，公元337-361年在位）在位初期所发行。正面铭文「DV CONSTANTINVS PT AVGG」——意即「神化君主君士坦丁，诸帝之父」——其中「PT」（Pater，之父）是追思币特有的称号，标明逝者为在位诸帝之父。戴维露姆面纱（velum）的半身像表明君士坦丁已被纳入神之行列。**特别值得关注的是正面铭文采用「DV」而非常见的「DN」（Dominus Noster，吾主）**——此或为特定造币厂之变体写法，亦可能因实物磨损导致字母辨识存疑，故仍以实物记录为准。 背面的「VN-MR」铭文实为「Veneranda Memoria」（应受崇敬之记忆）之缩写，是君士坦丁追思币中**特殊变体类型**之一。相较于更为常见的「CONS（Consecratio）」型封神图案（祭坛配阶梯），VN-MR型以**戴面纱穿托加的君士坦丁站姿全身像**为核心，配合「应受崇敬之记忆」的铭文，传达对已故君主的永恒怀念。底注「CONST」指示该币铸造于**君士坦丁堡造币厂**（Constantinople Mint），即君士坦丁大帝亲手建立的新都城。</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>2026-07-06T17:05:31</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add ROM-006: Hadrian LIBERALITAS AVG Sestertius, G/VG, raw patina, ¥370
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z21"/>
+  <dimension ref="A1:Z22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:30</t>
+          <t>2026-07-06T17:17:27</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:27</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:27</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:27</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
+          <t>2026-07-06T17:17:28</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,6 @@
           <t>私洽</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2778,11 +2777,125 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-06T17:05:31</t>
-        </is>
-      </c>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="inlineStr"/>
+          <t>2026-07-06T17:17:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ROM-006</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Liberalitas 慷慨女神赏赐型</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>哈德良 LIBERALITAS AVG 塞斯特提</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Liberalitas 慷慨女神赏赐型 · S C</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>AD 117-138</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Sestertius 塞斯特提</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Orichalcum 黄铜 · ~28mm · 19.93g</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>G/VG</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>roman</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>正面: 哈德良面向右之桂冠胸像 · 边缘环绕铭文（字迹受腐蚀覆盖）</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>背面: 坐姿Liberalitas女神像，右持计数板 · 铭文 LIBERALITAS AVG（皇帝之慷慨）· 底注 S C（Senatus Consulto，元老院决议）</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>罗马帝国, 哈德良, Liberalitas, 塞斯特提, 慷慨女神, congiarium, S C, 元老院, 1世纪末-2世纪, 2世纪, 生坑, 未清理</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>¥370</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>370</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>西西里晚祷</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>私洽</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>images/ROM-006.jpg</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>4884345</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>哈德良皇帝（Publius Aelius Hadrianus，公元117-138年在位）是一位以巡游帝国疆域、巩固边防和文化融合著称的「旅行皇帝」。在位期间，哈德良结束了前任图拉真大规模对外扩张的政策，转而巩固已有领土，重建犹太行省秩序，并以建筑伟大工程（万神殿重建、哈德良长城）闻名。 LIBERALITAS（慷慨女神）型塞斯特提是哈德良时期重要的政治宣传币种之一。此类型表现皇帝向民众分发赏赐（congiarium）的仪式场景——在位皇帝或代表坐在高处，向排队的公民分发钱币或实物。作为皇权与民众直接联系的重要仪式，congiarium既是皇恩浩荡的象征，也是元老院授权、皇权合法性的重要宣示。LIBERALITAS AVG型共有六个发行阶段（II-VI），分别对应不同年份的庆典赏赐：II为公元119年、III为121-122年、IV为125-126年、V为128年、VI为136年。 此枚金币正面为哈德良桂冠胸像，边缘环绕铭文（字迹受腐蚀和包浆覆盖，难以完整辨识）。背面为坐姿Liberalitas女神像，右侧手持计数板（abacus），场景上方铭文LIBERALITAS AVG，底注S C（Senatus Consulto，元老院决议）。 此币为未经清理的生坑状态，表面保留厚重原始包浆（绿锈+土黄沉积物），品相约G/VG。虽图录标注19.93g，目测接近典型塞斯特提标准重量（24-27g），可能存在出土后轻微失重。品相差但历史意义完整，¥370为合理捡漏价格。</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>2026-07-06T17:17:28</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add ROM-007: 1811 Napoleon Italy Kingdom 1 Soldo copper coin, NGC-AU50, ¥992
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z22"/>
+  <dimension ref="A1:Z23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:02</t>
+          <t>2026-07-06T17:40:33</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:02</t>
+          <t>2026-07-06T17:40:33</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:02</t>
+          <t>2026-07-06T17:40:33</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:02</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:02</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:02</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:02</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:02</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:02</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
+          <t>2026-07-06T17:40:34</t>
         </is>
       </c>
     </row>
@@ -2870,7 +2870,6 @@
           <t>私洽</t>
         </is>
       </c>
-      <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2886,16 +2885,130 @@
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>哈德良皇帝（Publius Aelius Hadrianus，公元117-138年在位）是一位以巡游帝国疆域、巩固边防和文化融合著称的「旅行皇帝」。在位期间，哈德良结束了前任图拉真大规模对外扩张的政策，转而巩固已有领土，重建犹太行省秩序，并以建筑伟大工程（万神殿重建、哈德良长城）闻名。 LIBERALITAS（慷慨女神）型塞斯特提是哈德良时期重要的政治宣传币种之一。此类型表现皇帝向民众分发赏赐（congiarium）的仪式场景——在位皇帝或代表坐在高处，向排队的公民分发钱币或实物。作为皇权与民众直接联系的重要仪式，congiarium既是皇恩浩荡的象征，也是元老院授权、皇权合法性的重要宣示。LIBERALITAS AVG型共有六个发行阶段（II-VI），分别对应不同年份的庆典赏赐：II为公元119年、III为121-122年、IV为125-126年、V为128年、VI为136年。 正面为哈德良面向右之桂冠胸像，赤裸上身，左肩披托加（toga），边缘环绕铭文「IMP CAESAR TRAIANVS HADRIANVS AVG」（最高统帅、凯撒·图拉真·哈德良·奥古斯都）。背面为皇帝赏赐场景（Congiarium）——哈德良坐在高台折叠椅（sella curulis）上，面左，右手前伸；助手向台下排队公民分发赏赐；慷慨女神Liberalitas站于背景处，手持钱袋（丘囊），场景上方铭文「PONT MAX TR POT COS II」，横书「LIBERALITAS AVG」，底注「S C」（Senatus Consulto，元老院决议）。 此币为未经清理的生坑状态，表面保留厚重原始包浆（绿锈+土黄沉积物），品相约G/VG。虽图录标注19.93g，目测接近典型塞斯特提标准重量（24-27g），可能存在出土后轻微失重。品相差但历史意义完整，¥370为合理捡漏价格。</t>
+          <t>在古罗马，有一种特殊的活动叫congiarium，起初它是向罗马城市居民分发油或酒，到奥古斯都时期演变成了在特殊场合（如皇帝登基、庆祝凯旋等）分发钱财。从尼禄统治时期开始，钱币上就出现了congiarium的场景，画面中总有一个人高举着带长柄的矩形物体。而当「慷慨」（Liberalitas）这一拟人形象在哈德良统治时期首次出现在钱币上时，这个矩形物体成了她的标志性特征。 这个神秘的矩形物体到底是什么呢？此前有多种解读。有人认为它是「tessera」（一种代币或凭证），也有人觉得是「abacus」（算盘），但观察不同皇帝时期钱币上对congiarium仪式图案的演变，尼禄时期的钱币上有两种图案形式，一种成了后续皇帝钱币的标准样式；图拉真时期的图案似乎印证congiarium有两个阶段；哈德良时期，「慷慨」拟人形象出现，逐渐取代了原本拿着矩形物体的男性形象。 结合历史记载中 congiarium 发放的货币面额信息（大多为第纳里乌斯银币，有时也会使用奥里斯金币），这个矩形物体极有可能是用于分发钱币的计数板。其表面的圆形凹陷，可辅助工作人员迅速数出待分发的钱币数量。在君士坦丁凯旋门的浮雕上，我们能够清晰看到皇帝使用类似物体向接受者分发钱币的场景。此外，画面中拿着它的人将其举到与头平齐或更高的位置展示给接受者和在场众人，保证分发过程的公平和诚实，避免出现盗窃和欺诈行为。 总的来说，这个成为「慷慨」拟人形象标志性特征的矩形物体，是congiarium仪式中不可或缺的计数、展示和分发工具，它在加快分发速度的同时，保障了分发的公正性。对于古罗马钱币收藏者而言，了解这些知识，能让我们手中的钱币「开口说话」，也是探索古罗马社会经济、政治和文化的重要线索。</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-06T17:21:03</t>
-        </is>
-      </c>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
+          <t>2026-07-06T17:40:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ROM-007</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>伦巴第铁王冠</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>拿破仑皇帝兼意大利国王1索尔迪铜币</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>伦巴第铁王冠 · 米兰造币厂</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>AD 1811</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>1 Soldo 索尔迪</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Copper 铜 · 22mm · ~4.6g</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>NGC-AU50</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>roman</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>正面: 拿破仑面向左之桂冠头像 · 铭文 NAPOLEONE IMPERATORE E RE（拿破仑皇帝兼国王）· 底部署名 1811 · 造币厂标记 M（Milano，米兰）</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>背面: 伦巴第铁王冠（Lombardy Iron Crown）· 顶部铭文 REGNO D'ITALIA（意大利王国）· 底部面值 1 SOLDO</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>拿破仑, 意大利王国, 拿破仑帝国, 索尔迪, 伦巴第铁王冠, 米兰, 19世纪, 1800-1815, NGC, 铜币, 意大利统一运动</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>¥992</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>992</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>云台主人</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>私洽</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>images/ROM-007.jpg</t>
+        </is>
+      </c>
+      <c r="V23" t="n">
+        <v>1700919</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>1811年拿破仑帝国鼎盛时期，意大利王国（Regno d'Italia）铸造的1索尔迪铜币。米兰造币厂（Mint Mark M）出品，编号NGC-AU50，成交价992元，来源云台主人2025年10月。 拿破仑于1805年在米兰加冕为意大利国王，随后在意大利领土上推行与法兰西帝国一致的行政、金融与货币体系。意大利王国使用法国货币标准：里拉（Lira）为记账单位，辅币包括索尔迪（Soldo，1里拉=20索尔迪）和分（Centesimo，1索尔迪=5分）。此枚1索尔迪铜币正面为拿破仑桂冠头像，铭文NAPOLEONE IMPERATORE E RE（拿破仑皇帝兼国王），底部署名1811与造币厂标记M（Milano）。背面为伦巴第铁王冠（Lombardy Iron Crown）——意大利统一运动的核心象征，王冠中心铭刻REGNO D'ITALIA（意大利王国），底部面值1 SOLDO。 伦巴第铁王冠（Lombardy Iron Crown）相传以钉死耶稣的圣钉铸造，直径4.5厘米，重约250克，外包金箔，内环为铁质。它是中世纪伦巴第王国及意大利独立运动的重要象征，拿破仑在取得马伦戈战役（1800年）后于伦巴第加冕时使用过此王冠。将铁王冠图案铸于钱币，既是拿破仑宣示其意大利王权的政治行为，也暗示他继承了意大利乃至神圣罗马帝国的历史正统性。此币NGC AU50品相，币面光亮，边齿锐利，是意大利王国拿破仑时期铜币的典型收藏品。</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>2026-07-06T17:40:34</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add NI-001: 1811 Napoleon Italy Kingdom 1 Soldo copper (Napoleon series)
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z23"/>
+  <dimension ref="A1:Z24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:33</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:33</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:33</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:23</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:24</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:24</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:24</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:24</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:24</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:24</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:24</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:24</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
+          <t>2026-07-06T17:43:24</t>
         </is>
       </c>
     </row>
@@ -2983,7 +2983,6 @@
           <t>私洽</t>
         </is>
       </c>
-      <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr">
         <is>
           <t>2025</t>
@@ -2994,9 +2993,6 @@
           <t>images/ROM-007.jpg</t>
         </is>
       </c>
-      <c r="V23" t="n">
-        <v>1700919</v>
-      </c>
       <c r="W23" t="inlineStr">
         <is>
           <t>1811年拿破仑帝国鼎盛时期，意大利王国（Regno d'Italia）铸造的1索尔迪铜币。米兰造币厂（Mint Mark M）出品，编号NGC-AU50，成交价992元，来源云台主人2025年10月。 拿破仑于1805年在米兰加冕为意大利国王，随后在意大利领土上推行与法兰西帝国一致的行政、金融与货币体系。意大利王国使用法国货币标准：里拉（Lira）为记账单位，辅币包括索尔迪（Soldo，1里拉=20索尔迪）和分（Centesimo，1索尔迪=5分）。此枚1索尔迪铜币正面为拿破仑桂冠头像，铭文NAPOLEONE IMPERATORE E RE（拿破仑皇帝兼国王），底部署名1811与造币厂标记M（Milano）。背面为伦巴第铁王冠（Lombardy Iron Crown）——意大利统一运动的核心象征，王冠中心铭刻REGNO D'ITALIA（意大利王国），底部面值1 SOLDO。 伦巴第铁王冠（Lombardy Iron Crown）相传以钉死耶稣的圣钉铸造，直径4.5厘米，重约250克，外包金箔，内环为铁质。它是中世纪伦巴第王国及意大利独立运动的重要象征，拿破仑在取得马伦戈战役（1800年）后于伦巴第加冕时使用过此王冠。将铁王冠图案铸于钱币，既是拿破仑宣示其意大利王权的政治行为，也暗示他继承了意大利乃至神圣罗马帝国的历史正统性。此币NGC AU50品相，币面光亮，边齿锐利，是意大利王国拿破仑时期铜币的典型收藏品。</t>
@@ -3004,11 +3000,123 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-07-06T17:40:34</t>
-        </is>
-      </c>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
+          <t>2026-07-06T17:43:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NI-001</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>伦巴第铁王冠</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>拿破仑皇帝兼意大利国王1索尔迪铜币</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>伦巴第铁王冠 · 米兰造币厂</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>AD 1811</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>1 Soldo 索尔迪</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Copper 铜 · 22mm · ~4.6g</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>NGC-AU50</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>napoleon-italy</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>正面: 拿破仑面向左之桂冠头像 · 铭文 NAPOLEONE IMPERATORE E RE（拿破仑皇帝兼国王）· 底部署名 1811 · 造币厂标记 M（Milano，米兰）</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>背面: 伦巴第铁王冠（Lombardy Iron Crown）· 顶部铭文 REGNO D'ITALIA（意大利王国）· 底部面值 1 SOLDO</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>拿破仑, 意大利王国, 拿破仑帝国, 索尔迪, 伦巴第铁王冠, 米兰, 19世纪, 1800-1815, NGC, 铜币, 意大利统一运动</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>¥992</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>992</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>云台主人</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>私洽</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>images/ROM-007.jpg</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>1811年拿破仑帝国鼎盛时期，意大利王国（Regno d'Italia）铸造的1索尔迪铜币。米兰造币厂（Mint Mark M）出品，编号NGC-AU50，成交价992元，来源云台主人2025年10月。 拿破仑于1805年在米兰加冕为意大利国王，随后在意大利领土上推行与法兰西帝国一致的行政、金融与货币体系。意大利王国使用法国货币标准：里拉（Lira）为记账单位，辅币包括索尔迪（Soldo，1里拉=20索尔迪）和分（Centesimo，1索尔迪=5分）。此枚1索尔迪铜币正面为拿破仑桂冠头像，铭文NAPOLEONE IMPERATORE E RE（拿破仑皇帝兼国王），底部署名1811与造币厂标记M（Milano）。背面为伦巴第铁王冠（Lombardy Iron Crown）——意大利统一运动的核心象征，王冠中心铭刻REGNO D'ITALIA（意大利王国），底部面值1 SOLDO。 伦巴第铁王冠（Lombardy Iron Crown）相传以钉死耶稣的圣钉铸造，直径4.5厘米，重约250克，外包金箔，内环为铁质。它是中世纪伦巴第王国及意大利独立运动的重要象征，拿破仑在取得马伦戈战役（1800年）后于伦巴第加冕时使用过此王冠。将铁王冠图案铸于钱币，既是拿破仑宣示其意大利王权的政治行为，也暗示他继承了意大利乃至神圣罗马帝国的历史正统性。此币NGC AU50品相，币面光亮，边齿锐利，是意大利王国拿破仑时期铜币的典型收藏品。</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>2026-07-06T17:43:24</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
delete ROM-007 (renamed to NI-001, Napoleon Italy series)
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:38</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:23</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:24</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:24</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:24</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:24</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:24</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:24</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:24</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:24</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:24</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3112,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:24</t>
+          <t>2026-07-06T17:45:39</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr"/>

</xml_diff>

<commit_message>
add GR-002: Istros Staters double heads silver, BC 340-313, £270
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z24"/>
+  <dimension ref="A1:Z25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:38</t>
+          <t>2026-07-07T14:51:02</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
+          <t>2026-07-07T14:51:03</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3093,6 @@
           <t>私洽</t>
         </is>
       </c>
-      <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr">
         <is>
           <t>2025</t>
@@ -3101,10 +3100,12 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>images/ROM-007.jpg</t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr"/>
+          <t>images/NI-001.jpg</t>
+        </is>
+      </c>
+      <c r="V24" t="n">
+        <v>1700919</v>
+      </c>
       <c r="W24" t="inlineStr">
         <is>
           <t>1811年拿破仑帝国鼎盛时期，意大利王国（Regno d'Italia）铸造的1索尔迪铜币。米兰造币厂（Mint Mark M）出品，编号NGC-AU50，成交价992元，来源云台主人2025年10月。 拿破仑于1805年在米兰加冕为意大利国王，随后在意大利领土上推行与法兰西帝国一致的行政、金融与货币体系。意大利王国使用法国货币标准：里拉（Lira）为记账单位，辅币包括索尔迪（Soldo，1里拉=20索尔迪）和分（Centesimo，1索尔迪=5分）。此枚1索尔迪铜币正面为拿破仑桂冠头像，铭文NAPOLEONE IMPERATORE E RE（拿破仑皇帝兼国王），底部署名1811与造币厂标记M（Milano）。背面为伦巴第铁王冠（Lombardy Iron Crown）——意大利统一运动的核心象征，王冠中心铭刻REGNO D'ITALIA（意大利王国），底部面值1 SOLDO。 伦巴第铁王冠（Lombardy Iron Crown）相传以钉死耶稣的圣钉铸造，直径4.5厘米，重约250克，外包金箔，内环为铁质。它是中世纪伦巴第王国及意大利独立运动的重要象征，拿破仑在取得马伦戈战役（1800年）后于伦巴第加冕时使用过此王冠。将铁王冠图案铸于钱币，既是拿破仑宣示其意大利王权的政治行为，也暗示他继承了意大利乃至神圣罗马帝国的历史正统性。此币NGC AU50品相，币面光亮，边齿锐利，是意大利王国拿破仑时期铜币的典型收藏品。</t>
@@ -3112,11 +3113,125 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-06T17:45:39</t>
-        </is>
-      </c>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
+          <t>2026-07-07T14:51:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GR-002</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>海鹰抓海豚</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>伊斯特罗斯 双人头银币</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>海鹰抓海豚 · 黑海古典银币</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>BC 340-BC 313</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Stater 斯塔特</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Silver 银 · 20.5mm · 5.53g</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>GVF</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>AMNG I-436; SNG BM Black Sea-237</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>greek</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>正面: 双少年头像 · 一正一反相互环绕 · 古典希腊城邦风格</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>背面: 海鹰展开双翅向左飞行抓握海豚 · 底部铭文 IΣTPIH（Istros，伊斯特罗斯）</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>希腊古典时期, 伊斯特罗斯, 莫西亚, 黑海殖民城邦, 双人头, 银币, 斯塔特, 古典时期, AMNG, SNG</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>£270</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>2484</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Classical Numismatic Group</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>拍卖</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>images/GR-002.jpg</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>289494</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>莫西亚（Moesia）伊斯特罗斯（Istros，黑海西岸重要城邦，约今罗马尼亚境内多瑙河三角洲）铸造的古典银币。 正面为双少年头像——一正一反、相互环绕。这种独特的双人头像图案是伊斯特罗斯城币的标志性设计，其象征意义学界尚有争议：一种观点认为代表Dioscuri（双子神卡斯托尔与波吕克斯），另一观点认为表现城邦的两位创建英雄或神灵（Heroes）。 背面为海鹰（鸥鹭）展开双翅抓握海豚，向左飞行。底部署名IΣTPIH（伊斯特罗斯城的希腊文名称）。这一图案反映了伊斯特罗斯作为黑海贸易港口的海洋经济特征——海鹰象征天空与神意，海豚象征海洋与商业繁荣，两者结合宣示城市对黑海贸易通道的掌控。 伊斯特罗斯城约公元前656年由米勒图斯（Miletus）移民建立，是黑海地区最早的希腊殖民城邦之一。其钱币铸造传统延续数百年，银币体系与雅典、爱奥尼亚等地有密切往来。</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>2026-07-07T14:51:04</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
migrate GK-005 to GR-003: Aspendos Staters (BC 380-325 → GR by BC 323 rule)
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z25"/>
+  <dimension ref="A1:Z26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:02</t>
+          <t>2026-07-07T14:57:52</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1893,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2438,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2777,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
     </row>
@@ -3227,11 +3227,114 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:04</t>
+          <t>2026-07-07T14:57:53</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>GR-003</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>GREECE</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>阿斯潘多斯 银质斯塔特</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>GREECE · Pamphylia · Aspendos (BC 380-325)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>BC 380-325</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Stater 斯塔特</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Silver 银 · 10.48g · 22mm</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>SNG France 103</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>greek</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>正面: 两名摔跤手搏斗 · "FK" 造币标记</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>背面: 投石手右行发射石弹 · triskeles · ΕΣΤΦΕΔΙΥΣ · pellet方框内</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>潘菲利亚, 阿斯潘多斯, 斯塔特</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>US$345</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>2484</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Aegean Numismatics</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>images/GR-003.jpg</t>
+        </is>
+      </c>
+      <c r="V26" t="n">
+        <v>112563</v>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>阿斯潘多斯（Aspendos）是潘菲利亚（Pamphylia）地区最重要的希腊殖民城市之一，位于欧里梅顿河（Eurymedon）入海口附近。该城在公元前 5 世纪波斯统治时期及随后的希腊化时期始终保持高度自治权，其独特的货币体系在整个安纳托利亚南部具有代表性。&lt;br&gt;&lt;br&gt;阿斯潘多斯银币正面描绘两名摔跤手（wrestlers）正在进行角力比赛——这是古希腊体育竞技（pankration 或 wrestling）的经典题材，可能与当地举办的运动赛事或狄奥斯库里（Dockeroi）的神话典故有关。两摔跤手之间的 "FK" 是造币厂缩写或工匠标记。&lt;br&gt;&lt;br&gt;背面描绘一名投石手（slinger）向右行走，正准备发射投石弹丸（bullet）。投石兵是安纳托利亚南部轻装步兵的典型代表，该形象可能与当地军事传统或赫拉克勒斯使用投石带的神话主题有关。三曲腿图（triskeles）是阿斯潘多斯币的典型辅助符号。铭文 "EΣTFEΔΙΙΥΣ" 是阿斯潘多斯（Aspendos）的希腊语城市名，置于颗粒方框（pellet square）内是潘菲利亚地区造币的典型边框设计。SNG France 103 将该版式归为阿斯潘多斯古典晚期（约 BC 380-325）标准银币。币面投石手下方有小凹痕（small ding below slinger）。</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>2026-07-07T14:57:53</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
gk renumber: reorder GK-001~010 by historical importance (Alexander first)
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z26"/>
+  <dimension ref="A1:Z27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:52</t>
+          <t>2026-07-07T15:40:27</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -815,42 +815,42 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PONTUS</t>
+          <t>GREECE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>本都·阿米索斯 珀尔修斯 / 飞马铜币</t>
+          <t>吕西马科斯 Lampsakos 四德拉克马</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PONTUS · Amisos · Mithradates VI Eupator</t>
+          <t>GREECE · Hellenistic · Lysimachos (BC 297-281)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>c. BC 85-65</t>
+          <t>BC 297-281</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AE 青铜</t>
+          <t>Tetradrachm 四德拉克马</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>AE 青铜 · 22mm · 11.38g · 轴 12h</t>
+          <t>Silver 银 · 28mm · 17.05g</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>gVF</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Waddington RG 32; cf. SNG BM Black Sea 1212-1217</t>
+          <t>Thompson 50; HGC 3 1750b</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -860,22 +860,22 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>正面: 珀尔修斯右向头像，戴弗里吉亚帽（狮鹫装饰）；Aegis 护符</t>
+          <t>正面: ΑΛΕΞΑΝΔΡΟΥ · 亚历山大大帝戴阿蒙（Ammon）角状头饰头像右</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>背面: ΑΜΙΣΟΥ · 飞马 Pegasus 左向饮水；exergue 内徽记</t>
+          <t>背面: ΑΘΗΝΑ · 雅典娜戴盔持盾矛立像右 · ΒΑΣΙΛΕΩΣ ΛΥΣΙΜΑΧΟΥ · ΑΘΗΝΑΣ（造币厂控制标记）</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>本都, 阿米索斯, 米特拉达梯六世, 珀尔修斯神话, 希腊化王国</t>
+          <t>希腊化, 吕西马科斯, Lampsakos, 亚历山大继承者</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>€35</t>
+          <t>€1,850</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -884,21 +884,11 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>273</v>
+        <v>14430</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Biga Numismatics</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Online Auction 38</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>2025</t>
+          <t>Camerarius Numizmatika</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -907,16 +897,16 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>138797</v>
+        <v>569494</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>本都（Pontus）是黑海南岸的希腊化王国，以阿米索斯（Amisos，今土耳其Samsun）为重要造币与商业中心。米特拉达梯六世（&lt;b&gt;Mithradates VI Eupator&lt;/b&gt;，约 120-63 BC）是本都最伟大的国王，史称"米特拉达梯大帝"——先后三次发动对罗马的战争（前 88-前 63 年"米特拉达梯战争"），一度征服小亚细亚、希腊和爱琴海诸岛，几乎推翻罗马在东方的霸权。最终被庞培击败，逃往克里米亚后自杀。&lt;br&gt;&lt;br&gt;此币的&lt;b&gt;珀尔修斯戴弗里吉亚帽（Pileus / Phrygian cap）&lt;/b&gt;形象有强烈的政治神话含义：米特拉达梯王室自诩为希腊英雄珀尔修斯（斩杀美杜莎、救赎安德洛墨达）后裔——珀尔修斯之子&lt;b&gt;Perses&lt;/b&gt;被认为波斯与本都王族的始祖。弗里吉亚帽在希腊罗马语境中象征&lt;b&gt;自由&lt;/b&gt;，而帽上的&lt;b&gt;狮鹫装饰（griffin-crest）&lt;/b&gt;则呼应波斯/东方传统，体现米特拉达梯横跨东西方的统治合法性。&lt;br&gt;&lt;br&gt;背面的&lt;b&gt;飞马 Pegasus&lt;/b&gt;是阿米索斯建城神话的核心元素（飞马用蹄踢出 Hippene 泉），也是该城数百年来的固定币面主题。这枚铜币是希腊化王国政治宣传与地方传统结合的典型样本。</t>
+          <t>吕西马科斯（Lysimachos，BC 360-281）是亚历山大大帝的六位近身侍卫（Somatophylax）之一，于BC 306/305年在色雷斯自立为王，建都莱普提昂杜斯（Lysimotelia），随后在其治下的色雷斯及小亚细亚地区大规模铸造四德拉克马金币。Lampsakos（兰普萨科斯）位于达达尼尔海峡入口，是吕西马科斯王国最重要的造币中心之一，掌控着从本都-潘提卡彭至爱琴海的贵金属流通命脉。&lt;br&gt;&lt;br&gt;吕西马科斯四德拉克马正面沿用经典的亚历山大阿蒙之角（Ammon Horn）形象——这一肖像自BC 336年起便随亚历山大的军事扩张流通于整个希腊化世界，是最早、最具辨识度的希腊化君主肖像。亚历山大通过宣称自己是埃及阿蒙神之子（Jupiter Ammon）来建构其神性血统，吕西马科斯沿用这一肖像，既是政治宣传，也是对亚历山大开创的希腊化君主制iconography（肖像体系）的直接继承。&lt;br&gt;&lt;br&gt;背面雅典娜·阿尔基德莫斯（Athena Alkidemos）是马其顿及亚历山大继承者们偏爱的战神形象——手持阿尔基（Alche，阿克顿的神盾）和矛，身披盔甲配狮皮头盔。Lampsakos造币厂以ΑΘΗΝΑΣ作为控制标记（control mark），用于区分不同批次和工匠。吕西马科斯四德拉克马是希腊化时期发行量最大、流通最广的硬币版式之一。</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1019,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1132,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1245,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1358,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -1380,42 +1370,42 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GREECE</t>
+          <t>SELEUCID EMPIRE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>吕西马科斯 Lampsakos 四德拉克马</t>
+          <t>塞琉古帝国塞琉古一世铜币</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>GREECE · Hellenistic · Lysimachos (BC 297-281)</t>
+          <t>SELEUCID EMPIRE · ELEPHANT &amp; BUCERAS</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BC 297-281</t>
+          <t>公元前312-前281年</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Tetradrachm 四德拉克马</t>
+          <t>Chalkous 铜币</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Silver 银 · 28mm · 17.05g</t>
+          <t>Bronze 青铜 · 22mm · 6.42g</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>gVF</t>
+          <t>VF</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Thompson 50; HGC 3 1750b</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1425,35 +1415,45 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>正面: ΑΛΕΞΑΝΔΡΟΥ · 亚历山大大帝戴阿蒙（Ammon）角状头饰头像右</t>
+          <t>正面: 亚洲象向右行走 · 体态健壮 · 背上驮有辎重</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>背面: ΑΘΗΝΑ · 雅典娜戴盔持盾矛立像右 · ΒΑΣΙΛΕΩΣ ΛΥΣΙΜΑΧΟΥ · ΑΘΗΝΑΣ（造币厂控制标记）</t>
+          <t>背面: 戴牛角之马头向右 · 下方船锚 ⚓ · 铭文 ΒΑΣΙΛΕΩΣ ΣΕΛΕΥΚΟΥ</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>希腊化, 吕西马科斯, Lampsakos, 亚历山大继承者</t>
+          <t>塞琉古, 塞琉古一世, 胜利者, Nikator, 亚洲象, 布克法罗斯, Bucephalus, 阿帕美亚, 伊普苏斯, 继业者战争, 船锚</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>€1,850</t>
+          <t>¥360</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="P9" t="n">
-        <v>14430</v>
+        <v>360</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Camerarius Numizmatika</t>
+          <t>西西里晚祷</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>私洽</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1462,16 +1462,16 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>569494</v>
+        <v>175619</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>吕西马科斯（Lysimachos，BC 360-281）是亚历山大大帝的六位近身侍卫（Somatophylax）之一，于BC 306/305年在色雷斯自立为王，建都莱普提昂杜斯（Lysimotelia），随后在其治下的色雷斯及小亚细亚地区大规模铸造四德拉克马金币。Lampsakos（兰普萨科斯）位于达达尼尔海峡入口，是吕西马科斯王国最重要的造币中心之一，掌控着从本都-潘提卡彭至爱琴海的贵金属流通命脉。&lt;br&gt;&lt;br&gt;吕西马科斯四德拉克马正面沿用经典的亚历山大阿蒙之角（Ammon Horn）形象——这一肖像自BC 336年起便随亚历山大的军事扩张流通于整个希腊化世界，是最早、最具辨识度的希腊化君主肖像。亚历山大通过宣称自己是埃及阿蒙神之子（Jupiter Ammon）来建构其神性血统，吕西马科斯沿用这一肖像，既是政治宣传，也是对亚历山大开创的希腊化君主制iconography（肖像体系）的直接继承。&lt;br&gt;&lt;br&gt;背面雅典娜·阿尔基德莫斯（Athena Alkidemos）是马其顿及亚历山大继承者们偏爱的战神形象——手持阿尔基（Alche，阿克顿的神盾）和矛，身披盔甲配狮皮头盔。Lampsakos造币厂以ΑΘΗΝΑΣ作为控制标记（control mark），用于区分不同批次和工匠。吕西马科斯四德拉克马是希腊化时期发行量最大、流通最广的硬币版式之一。</t>
+          <t>公元前323年亚历山大大帝骤然离世，其帝国随即陷入继业者战争（War of the Diadochi）。塞琉古（Seleucus）作为亚历山大的近身护卫官，于公元前321年被迫流亡埃及。公元前312年，在托勒密一世的支持下，塞琉古重返巴比伦，宣布独立，开启了塞琉古帝国长达两百余年的统治，是年便成为塞琉古纪元的元年。公元前301年伊普苏斯战役（Battle of Ipsus），塞琉古与利西马科斯（Lysimachus）联手击败安提柯（Antigonus），瓜分亚历山大帝国的东部版图，塞琉古一跃成为从安纳托利亚延伸至印度的庞大帝国之君，领土面积仅次于孔雀王朝印度。 阿帕美亚（Apamaea on the Orontes）位于奥隆特斯河畔，是塞琉古帝国最繁华的城市之一，以其母——塞琉古一世之妻阿帕美亚（Apama）命名，与安条克、塞琉西亚并列为帝国三大都城。 此币正面亚洲象向右行走，象征塞琉古从印度孔雀王朝君主旃陀罗笈多（Chandragupta）手中换取的五百头战象，这些战象是伊普苏斯战役决定性胜利的关键；背面戴牛角之马头为布克法罗斯（Bucephalus）的形象，据传是亚历山大大帝的传奇坐骑，塞琉古以布克法罗斯自比，昭示其作为亚历山大正统继承人的身份；船锚则暗指塞琉古大腿根部形似锚状的胎记，同时也象征其祖先尼卡托尔（Nicator，意为「胜利者」）作为亚历山大海军指挥官与腓力二世时期的海军将领之出身，将希腊世界的海上传统与新帝国紧紧相连。</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -1483,32 +1483,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GREECE</t>
+          <t>MACEDON</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>阿斯潘多斯 银质斯塔特</t>
+          <t>腓力二世 青铜币</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>GREECE · Pamphylia · Aspendos (BC 380-325)</t>
+          <t>MACEDON · Philip II (359-336 BC)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BC 380-325</t>
+          <t>359-336 BC</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Stater 斯塔特</t>
+          <t>AE 青铜</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Silver 银 · 10.48g · 22mm</t>
+          <t>Bronze 青铜 · 6g · 17.3mm</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>SNG France 103</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1528,35 +1528,40 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>正面: 两名摔跤手搏斗 · "FK" 造币标记</t>
+          <t>正面: 阿波罗戴王冠头像右向</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>背面: 投石手右行发射石弹 · triskeles · ΕΣΤΦΕΔΙΥΣ · pellet方框内</t>
+          <t>背面: ΦΙΛΙΠΠΟΥ · 青年骑手立马右行立起</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>潘菲利亚, 阿斯潘多斯, 斯塔特</t>
+          <t>马其顿, 腓力二世, 亚历山大之父</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>US$345</t>
+          <t>¥369</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>2484</v>
+        <v>369</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Aegean Numismatics</t>
+          <t>凝绿轩</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>2024</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1565,16 +1570,16 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>112563</v>
+        <v>25477</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>阿斯潘多斯（Aspendos）是潘菲利亚（Pamphylia）地区最重要的希腊殖民城市之一，位于欧里梅顿河（Eurymedon）入海口附近。该城在公元前 5 世纪波斯统治时期及随后的希腊化时期始终保持高度自治权，其独特的货币体系在整个安纳托利亚南部具有代表性。&lt;br&gt;&lt;br&gt;阿斯潘多斯银币正面描绘两名摔跤手（wrestlers）正在进行角力比赛——这是古希腊体育竞技（pankration 或 wrestling）的经典题材，可能与当地举办的运动赛事或狄奥斯库里（Dockeroi）的神话典故有关。两摔跤手之间的 "FK" 是造币厂缩写或工匠标记。&lt;br&gt;&lt;br&gt;背面描绘一名投石手（slinger）向右行走，正准备发射投石弹丸（bullet）。投石兵是安纳托利亚南部轻装步兵的典型代表，该形象可能与当地军事传统或赫拉克勒斯使用投石带的神话主题有关。三曲腿图（triskeles）是阿斯潘多斯币的典型辅助符号。铭文 "EΣTFEΔΙΙΥΣ" 是阿斯潘多斯（Aspendos）的希腊语城市名，置于颗粒方框（pellet square）内是潘菲利亚地区造币的典型边框设计。SNG France 103 将该版式归为阿斯潘多斯古典晚期（约 BC 380-325）标准银币。币面投石手下方有小凹痕（small ding below slinger）。</t>
+          <t>腓力二世（Philip II）是马其顿王国国王（公元前359-336年），亚历山大大帝之父。他通过军事改革（"马其顿方阵"战术创新）和外交手段，将马其顿从希腊边缘小国提升为希腊霸主，为亚历山大的帝国奠定基础。公元前338年喀罗尼亚战役击败希腊城邦联军后，腓力被尊为希腊世界实际统治者。&lt;br&gt;&lt;br&gt;腓力二世青铜币正面为阿波罗戴王冠头像，阿波罗是希腊神话中的太阳神和音乐之神，也是马其顿王室的重要保护神。背面为青年骑手图像，是马其顿王室标志性的 iconography，铭文"ΦΙΛΙΠΠΟΥ"（腓力普斯/腓力）标明发行者身份。这类青铜小币主要作为辅币流通，用于日常小额交易。</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:03</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -1586,22 +1591,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MACEDON</t>
+          <t>PONTUS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>腓力二世 青铜币</t>
+          <t>本都·阿米索斯 珀尔修斯 / 飞马铜币</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MACEDON · Philip II (359-336 BC)</t>
+          <t>PONTUS · Amisos · Mithradates VI Eupator</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>359-336 BC</t>
+          <t>c. BC 85-65</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1611,17 +1616,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Bronze 青铜 · 6g · 17.3mm</t>
+          <t>AE 青铜 · 22mm · 11.38g · 轴 12h</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>F</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Waddington RG 32; cf. SNG BM Black Sea 1212-1217</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1631,40 +1636,45 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>正面: 阿波罗戴王冠头像右向</t>
+          <t>正面: 珀尔修斯右向头像，戴弗里吉亚帽（狮鹫装饰）；Aegis 护符</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>背面: ΦΙΛΙΠΠΟΥ · 青年骑手立马右行立起</t>
+          <t>背面: ΑΜΙΣΟΥ · 飞马 Pegasus 左向饮水；exergue 内徽记</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>马其顿, 腓力二世, 亚历山大之父</t>
+          <t>本都, 阿米索斯, 米特拉达梯六世, 珀尔修斯神话, 希腊化王国</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>¥369</t>
+          <t>€35</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>CNY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>369</v>
+        <v>273</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>凝绿轩</t>
+          <t>Biga Numismatics</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Online Auction 38</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1673,16 +1683,16 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>25477</v>
+        <v>973582</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>腓力二世（Philip II）是马其顿王国国王（公元前359-336年），亚历山大大帝之父。他通过军事改革（"马其顿方阵"战术创新）和外交手段，将马其顿从希腊边缘小国提升为希腊霸主，为亚历山大的帝国奠定基础。公元前338年喀罗尼亚战役击败希腊城邦联军后，腓力被尊为希腊世界实际统治者。&lt;br&gt;&lt;br&gt;腓力二世青铜币正面为阿波罗戴王冠头像，阿波罗是希腊神话中的太阳神和音乐之神，也是马其顿王室的重要保护神。背面为青年骑手图像，是马其顿王室标志性的 iconography，铭文"ΦΙΛΙΠΠΟΥ"（腓力普斯/腓力）标明发行者身份。这类青铜小币主要作为辅币流通，用于日常小额交易。</t>
+          <t>本都（Pontus）是黑海南岸的希腊化王国，以阿米索斯（Amisos，今土耳其Samsun）为重要造币与商业中心。米特拉达梯六世（&lt;b&gt;Mithradates VI Eupator&lt;/b&gt;，约 120-63 BC）是本都最伟大的国王，史称"米特拉达梯大帝"——先后三次发动对罗马的战争（前 88-前 63 年"米特拉达梯战争"），一度征服小亚细亚、希腊和爱琴海诸岛，几乎推翻罗马在东方的霸权。最终被庞培击败，逃往克里米亚后自杀。&lt;br&gt;&lt;br&gt;此币的&lt;b&gt;珀尔修斯戴弗里吉亚帽（Pileus / Phrygian cap）&lt;/b&gt;形象有强烈的政治神话含义：米特拉达梯王室自诩为希腊英雄珀尔修斯（斩杀美杜莎、救赎安德洛墨达）后裔——珀尔修斯之子&lt;b&gt;Perses&lt;/b&gt;被认为波斯与本都王族的始祖。弗里吉亚帽在希腊罗马语境中象征&lt;b&gt;自由&lt;/b&gt;，而帽上的&lt;b&gt;狮鹫装饰（griffin-crest）&lt;/b&gt;则呼应波斯/东方传统，体现米特拉达梯横跨东西方的统治合法性。&lt;br&gt;&lt;br&gt;背面的&lt;b&gt;飞马 Pegasus&lt;/b&gt;是阿米索斯建城神话的核心元素（飞马用蹄踢出 Hippene 泉），也是该城数百年来的固定币面主题。这枚铜币是希腊化王国政治宣传与地方传统结合的典型样本。</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1800,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1903,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -1996,7 +2006,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2109,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -2111,22 +2121,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MACEDONIA</t>
+          <t>LAODIKEIA AD LYCUM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>马其顿·亚历山大三世 大帝 四德拉克马</t>
+          <t>弗里几亚劳迪西亚城·蛇篮式四德拉克马</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MACEDONIA · ALEXANDER III</t>
+          <t>LAODIKEIA AD LYCUM · SERPENT FROM CISTA MYSTICA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BC 336-323</t>
+          <t>公元前133-前67年</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2136,19 +2146,19 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Silver 银 · 26mm · 16.9g</t>
+          <t>Silver 银 · 27.5mm · 12.56g</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
           <t>greek</t>
@@ -2156,22 +2166,22 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>正面: 赫拉克勒斯狮皮盔头像</t>
+          <t>正面: 蛇正从篮中爬出，周围常春藤花环环绕，花叶饱满</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>背面: 宙斯持鹰坐像 · ΑΛΕΞΑΝΔΡΟΥ（亚历山大的）</t>
+          <t>背面: 两条蛇缠绕弓箭袋 · AΠOΛΛΩNIOΣ ΕΥΑΡΧΟΥ · 左下角ΛΑΟ</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>亚历山大, 希腊化, 四德, 马其顿, 赫拉克勒斯, 宙斯</t>
+          <t>蛇篮, 劳迪西亚, 弗里几亚, 罗马统治, 狄奥尼索斯, 常春藤</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>¥4,000</t>
+          <t>¥2,888</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -2180,11 +2190,11 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>4000</v>
+        <v>2888</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>达爷</t>
+          <t>熊太乐</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -2203,16 +2213,16 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>484438</v>
+        <v>3871047</v>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>亚历山大三世（大帝，356-323 BC）统一希腊、征服波斯，建立了人类历史上第一个横跨欧亚非的超级帝国。他对货币体系的改革影响深远：四德拉克马银币以赫拉克勒斯头像为正面，宙斯持鹰坐像为背面，成为帝国扩张的战略工具与文化符号。随着亚历山大的征服，这套币制被推广至从埃及到印度河的广大地区，继业者纷纷仿铸。利西普斯（ Lysippos ）风格的赫拉克勒斯肖像极具古典理想美，而宙斯坐像手持雄鹰的形象则强化了王权的神圣性。此枚米勒都斯（Miletus）铸币约 BC 325-320 年所见宙斯底座无碑铭，为亚历山大在世时期的早期铸型。</t>
+          <t>蛇篮（Cista Mystica）是古希腊祭祀酒神狄奥尼索斯仪式中的神圣器物——一个装有幼蛇的柳编篮子，祭司将其取出让蛇爬出，以此象征神迹与重生。这一意象被广泛铸造在银币背面，成为古希腊钱币中最具神秘感的经典图式。此币正面蛇从篮中爬出，周围常春藤花环环绕；背面双蛇缠绕弓箭袋，铭文「AΠOΛΛΩNIOΣ ΕΥΑΡΧΟΥ」清晰漂亮——地方行政官阿波罗尼奥斯，尤阿尔科斯之子。公元前133年帕加马王国灭亡，小亚细亚落入罗马人之手，此币恐由罗马总督发行，兑换比率为三枚狄纳里银币换一枚蛇篮四德拉克马。</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -2337,32 +2347,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LAODIKEIA AD LYCUM</t>
+          <t>CYRENE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>弗里几亚劳迪西亚城·蛇篮式四德拉克马</t>
+          <t>昔兰尼阿波罗-忘忧草2德拉克马</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>LAODIKEIA AD LYCUM · SERPENT FROM CISTA MYSTICA</t>
+          <t>CYRENE · APOLLO CARNEIUS &amp; SILPHIUM</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>公元前133-前67年</t>
+          <t>公元前294-前275年</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Tetradrachm 四德拉克马</t>
+          <t>Didrachm 2德拉克马</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Silver 银 · 27.5mm · 12.56g</t>
+          <t>Silver 银 · 19mm · 7.62g</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2382,22 +2392,22 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>正面: 蛇正从篮中爬出，周围常春藤花环环绕，花叶饱满</t>
+          <t>正面: 阿波罗·卡内奥斯（Apollo Carneius）侧面头像 · 年轻俊美 · 羊角与桂冠共存</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>背面: 两条蛇缠绕弓箭袋 · AΠOΛΛΩNIOΣ ΕΥΑΡΧΟΥ · 左下角ΛΑΟ</t>
+          <t>背面: Silphium忘忧草 · 茎粗壮 · 心形果实 · 卷曲根系</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>蛇篮, 劳迪西亚, 弗里几亚, 罗马统治, 狄奥尼索斯, 常春藤</t>
+          <t>昔兰尼, 阿波罗, 忘忧草, Silphium, 塞琉古, 罗马统治, 避孕, 灭绝植物</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>¥2,888</t>
+          <t>¥5,500</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -2406,7 +2416,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>2888</v>
+        <v>5500</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -2429,16 +2439,16 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>3871047</v>
+        <v>3492219</v>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>蛇篮（Cista Mystica）是古希腊祭祀酒神狄奥尼索斯仪式中的神圣器物——一个装有幼蛇的柳编篮子，祭司将其取出让蛇爬出，以此象征神迹与重生。这一意象被广泛铸造在银币背面，成为古希腊钱币中最具神秘感的经典图式。此币正面蛇从篮中爬出，周围常春藤花环环绕；背面双蛇缠绕弓箭袋，铭文「AΠOΛΛΩNIOΣ ΕΥΑΡΧΟΥ」清晰漂亮——地方行政官阿波罗尼奥斯，尤阿尔科斯之子。公元前133年帕加马王国灭亡，小亚细亚落入罗马人之手，此币恐由罗马总督发行，兑换比率为三枚狄纳里银币换一枚蛇篮四德拉克马。</t>
+          <t>昔兰尼（Cyrenaica，今利比亚东部）于公元前631年建城，相传由一群来自帖飞的移民在阿波罗神谕指引下建立。此城迅速崛起为古代世界最富庶的城邦之一，全赖一种神奇植物——Silphium（又名忘忧草， Laserpitium silphium）。这种形似巨大茴香的伞形科植物，只生长在昔兰尼周边海岸，拥有令人惊叹的医疗功效，尤其以高效的避孕作用闻名——古代妇女将其汁液涂抹于子宫口，成功率接近百分之百。其贸易价值极高，一磅Silphium的价格相当于一个罗马士兵六年的薪俸，罗马元老院甚至在其铸造的银币上压制Silphium图案，作为帝国繁荣的象征。塞琉古帝国在公元前3世纪初攻占昔兰尼后废止本地铸币，此币发行于城市沦陷后的罗马统治早期，由当地官员以原塞琉古模具或本地模具发行，正面阿波罗·卡内奥斯（Apollo Carneius，羊角神）头像，羊角与桂冠共存，象征城邦保护神的神圣权威；背面Silphium枝叶繁茂，茎粗壮有力，果实心脏形，根系卷曲——这一经典图式在昔兰尼钱币上延续了两百余年。令人唏嘘的是，公元1世纪Silphium已彻底灭绝，原因可能是过度采集、地震破坏与土壤退化三重打击。</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2787,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2900,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3123,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3237,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr"/>
@@ -3332,7 +3342,120 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T15:40:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>GK-001</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>MACEDONIA</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>马其顿·亚历山大三世 大帝 四德拉克马</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>MACEDONIA · ALEXANDER III</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>BC 336-323</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Tetradrachm 四德拉克马</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Silver 银 · 26mm · 16.9g</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>greek</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>正面: 赫拉克勒斯狮皮盔头像</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>背面: 宙斯持鹰坐像 · ΑΛΕΞΑΝΔΡΟΥ（亚历山大的）</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>亚历山大, 希腊化, 四德, 马其顿, 赫拉克勒斯, 宙斯</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>¥4,000</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>4000</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>达爷</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>私洽</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>images/GK-001.jpg</t>
+        </is>
+      </c>
+      <c r="V27" t="n">
+        <v>484438</v>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>亚历山大三世（大帝，356-323 BC）统一希腊、征服波斯，建立了人类历史上第一个横跨欧亚非的超级帝国。他对货币体系的改革影响深远：四德拉克马银币以赫拉克勒斯头像为正面，宙斯持鹰坐像为背面，成为帝国扩张的战略工具与文化符号。随着亚历山大的征服，这套币制被推广至从埃及到印度河的广大地区，继业者纷纷仿铸。利西普斯（ Lysippos ）风格的赫拉克勒斯肖像极具古典理想美，而宙斯坐像手持雄鹰的形象则强化了王权的神圣性。此枚米勒都斯（Miletus）铸币约 BC 325-320 年所见宙斯底座无碑铭，为亚历山大在世时期的早期铸型。</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>2026-07-07T15:40:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
GK-011: 实物图入库 + 修正obverse为Mithradates VI戴王缰带(non-winged)
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:27</t>
+          <t>2026-07-07T16:02:52</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -1591,42 +1591,42 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PONTUS</t>
+          <t>ATHENS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>本都·阿米索斯 珀尔修斯 / 飞马铜币</t>
+          <t>雅典城·新式猫头鹰 四德拉克马</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>PONTUS · Amisos · Mithradates VI Eupator</t>
+          <t>ATHENS · NEW STYLE OWL</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>c. BC 85-65</t>
+          <t>BC 2nd-1st Century</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AE 青铜</t>
+          <t>Tetradrachm 四德拉克马</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>AE 青铜 · 22mm · 11.38g · 轴 12h</t>
+          <t>Silver 银 · 31.6mm · 16.7g</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Waddington RG 32; cf. SNG BM Black Sea 1212-1217</t>
+          <t>—</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1636,40 +1636,40 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>正面: 珀尔修斯右向头像，戴弗里吉亚帽（狮鹫装饰）；Aegis 护符</t>
+          <t>正面: 雅典娜女神戴阿提卡式头盔头像</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>背面: ΑΜΙΣΟΥ · 飞马 Pegasus 左向饮水；exergue 内徽记</t>
+          <t>背面: 猫头鹰立于双耳陶罐上 · 橄榄枝环绕 · ΑΘΕ</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>本都, 阿米索斯, 米特拉达梯六世, 珀尔修斯神话, 希腊化王国</t>
+          <t>雅典, 猫头鹰, 希腊化, 四德, 雅典娜</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>€35</t>
+          <t>¥13,500</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>CNY</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>273</v>
+        <v>13500</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Biga Numismatics</t>
+          <t>大象古币</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Online Auction 38</t>
+          <t>私洽</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -1687,12 +1687,12 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>本都（Pontus）是黑海南岸的希腊化王国，以阿米索斯（Amisos，今土耳其Samsun）为重要造币与商业中心。米特拉达梯六世（&lt;b&gt;Mithradates VI Eupator&lt;/b&gt;，约 120-63 BC）是本都最伟大的国王，史称"米特拉达梯大帝"——先后三次发动对罗马的战争（前 88-前 63 年"米特拉达梯战争"），一度征服小亚细亚、希腊和爱琴海诸岛，几乎推翻罗马在东方的霸权。最终被庞培击败，逃往克里米亚后自杀。&lt;br&gt;&lt;br&gt;此币的&lt;b&gt;珀尔修斯戴弗里吉亚帽（Pileus / Phrygian cap）&lt;/b&gt;形象有强烈的政治神话含义：米特拉达梯王室自诩为希腊英雄珀尔修斯（斩杀美杜莎、救赎安德洛墨达）后裔——珀尔修斯之子&lt;b&gt;Perses&lt;/b&gt;被认为波斯与本都王族的始祖。弗里吉亚帽在希腊罗马语境中象征&lt;b&gt;自由&lt;/b&gt;，而帽上的&lt;b&gt;狮鹫装饰（griffin-crest）&lt;/b&gt;则呼应波斯/东方传统，体现米特拉达梯横跨东西方的统治合法性。&lt;br&gt;&lt;br&gt;背面的&lt;b&gt;飞马 Pegasus&lt;/b&gt;是阿米索斯建城神话的核心元素（飞马用蹄踢出 Hippene 泉），也是该城数百年来的固定币面主题。这枚铜币是希腊化王国政治宣传与地方传统结合的典型样本。</t>
+          <t>雅典猫头鹰银币是古希腊最具代表性的货币，从公元前5世纪延续至公元前1世纪，成为古代地中海世界的硬通货。古典时期结束后，雅典于公元前2世纪摆脱马其顿控制，重启银币铸造，采用全新设计风格——新式猫头鹰（New Style）。与古典版相比，新式猫头鹰正面雅典娜头像更为精致，头戴装饰丰富的阿提卡式头盔；背面猫头鹰立于双耳陶罐（amphora）之上，周边环绕橄榄枝，并刻有地方官姓名与徽记，体现了希腊化时期雅典城邦的自治与繁荣。</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -2234,42 +2234,42 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ATHENS</t>
+          <t>PONTUS</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>雅典城·新式猫头鹰 四德拉克马</t>
+          <t>本都·阿米索斯 珀尔修斯 / 飞马铜币</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ATHENS · NEW STYLE OWL</t>
+          <t>PONTUS · Amisos · Mithradates VI Eupator</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BC 2nd-1st Century</t>
+          <t>c. BC 85-65</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Tetradrachm 四德拉克马</t>
+          <t>AE 青铜</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Silver 银 · 31.6mm · 16.7g</t>
+          <t>AE 青铜 · 22mm · 11.38g · 轴 12h</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>F</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Waddington RG 32; cf. SNG BM Black Sea 1212-1217</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -2279,40 +2279,40 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>正面: 雅典娜女神戴阿提卡式头盔头像</t>
+          <t>正面: 珀尔修斯右向头像，戴弗里吉亚帽（狮鹫装饰）；Aegis 护符</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>背面: 猫头鹰立于双耳陶罐上 · 橄榄枝环绕 · ΑΘΕ</t>
+          <t>背面: ΑΜΙΣΟΥ · 飞马 Pegasus 左向饮水；exergue 内徽记</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>雅典, 猫头鹰, 希腊化, 四德, 雅典娜</t>
+          <t>本都, 阿米索斯, 米特拉达梯六世, 珀尔修斯神话, 希腊化王国</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>¥13,500</t>
+          <t>€35</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>CNY</t>
+          <t>EUR</t>
         </is>
       </c>
       <c r="P17" t="n">
-        <v>13500</v>
+        <v>273</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>大象古币</t>
+          <t>Biga Numismatics</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>私洽</t>
+          <t>Online Auction 38</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -2326,16 +2326,16 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>973582</v>
+        <v>138797</v>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>雅典猫头鹰银币是古希腊最具代表性的货币，从公元前5世纪延续至公元前1世纪，成为古代地中海世界的硬通货。古典时期结束后，雅典于公元前2世纪摆脱马其顿控制，重启银币铸造，采用全新设计风格——新式猫头鹰（New Style）。与古典版相比，新式猫头鹰正面雅典娜头像更为精致，头戴装饰丰富的阿提卡式头盔；背面猫头鹰立于双耳陶罐（amphora）之上，周边环绕橄榄枝，并刻有地方官姓名与徽记，体现了希腊化时期雅典城邦的自治与繁荣。</t>
+          <t>本都（Pontus）是黑海南岸的希腊化王国，以阿米索斯（Amisos，今土耳其Samsun）为重要造币与商业中心。米特拉达梯六世（&lt;b&gt;Mithradates VI Eupator&lt;/b&gt;，约 120-63 BC）是本都最伟大的国王，史称"米特拉达梯大帝"——先后三次发动对罗马的战争（前 88-前 63 年"米特拉达梯战争"），一度征服小亚细亚、希腊和爱琴海诸岛，几乎推翻罗马在东方的霸权。最终被庞培击败，逃往克里米亚后自杀。&lt;br&gt;&lt;br&gt;此币的&lt;b&gt;珀尔修斯戴弗里吉亚帽（Pileus / Phrygian cap）&lt;/b&gt;形象有强烈的政治神话含义：米特拉达梯王室自诩为希腊英雄珀尔修斯（斩杀美杜莎、救赎安德洛墨达）后裔——珀尔修斯之子&lt;b&gt;Perses&lt;/b&gt;被认为波斯与本都王族的始祖。弗里吉亚帽在希腊罗马语境中象征&lt;b&gt;自由&lt;/b&gt;，而帽上的&lt;b&gt;狮鹫装饰（griffin-crest）&lt;/b&gt;则呼应波斯/东方传统，体现米特拉达梯横跨东西方的统治合法性。&lt;br&gt;&lt;br&gt;背面的&lt;b&gt;飞马 Pegasus&lt;/b&gt;是阿米索斯建城神话的核心元素（飞马用蹄踢出 Hippene 泉），也是该城数百年来的固定币面主题。这枚铜币是希腊化王国政治宣传与地方传统结合的典型样本。</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -2460,108 +2460,115 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CYRENE</t>
+          <t>本都王国</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>昔兰尼阿波罗-忘忧草2德拉克马</t>
+          <t>本都·阿米索斯 米特里达梯六世/丰饶角铜币</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CYRENE · APOLLO CARNEIUS &amp; SILPHIUM</t>
+          <t>本都王国·米特里达梯六世摄政时期</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>公元前294-前275年</t>
+          <t>约BC 120-BC 100</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Didrachm 2德拉克马</t>
+          <t>AE18</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Silver 银 · 19mm · 7.62g</t>
+          <t>青铜 · 18mm · 4.37g</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>Good Very Fine; gentle shimmer to surface</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SNG Stancomb-668; SNG France-1129-33; HGC 7-249</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>greek</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>正面: 阿波罗·卡内奥斯（Apollo Carneius）侧面头像 · 年轻俊美 · 羊角与桂冠共存</t>
+          <t>正面: 米特里达梯六世戴王缰带头向右胸像</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>背面: Silphium忘忧草 · 茎粗壮 · 心形果实 · 卷曲根系</t>
+          <t>背面: 丰饶角两侧为狄俄斯库里兄弟皮里帽，ΑΜΙ-ΣΟΥ横列下方</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>昔兰尼, 阿波罗, 忘忧草, Silphium, 塞琉古, 罗马统治, 避孕, 灭绝植物</t>
+          <t>本都, 阿米索斯, 丰饶角, 狄俄斯库里, 希腊化, 米特里达梯六世, 米特里达梯王朝</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>¥5,500</t>
+          <t>£36</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>CNY</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="P19" t="n">
-        <v>5500</v>
+        <v>331</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>熊太乐</t>
+          <t>The Coin CABINET</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>私洽</t>
-        </is>
-      </c>
+          <t>Auction Ancients 34</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>images/GK-011.jpg</t>
+          <t>images/gk-011.jpg</t>
         </is>
       </c>
       <c r="V19" t="n">
-        <v>3492219</v>
+        <v>302838</v>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>昔兰尼（Cyrenaica，今利比亚东部）于公元前631年建城，相传由一群来自帖飞的移民在阿波罗神谕指引下建立。此城迅速崛起为古代世界最富庶的城邦之一，全赖一种神奇植物——Silphium（又名忘忧草， Laserpitium silphium）。这种形似巨大茴香的伞形科植物，只生长在昔兰尼周边海岸，拥有令人惊叹的医疗功效，尤其以高效的避孕作用闻名——古代妇女将其汁液涂抹于子宫口，成功率接近百分之百。其贸易价值极高，一磅Silphium的价格相当于一个罗马士兵六年的薪俸，罗马元老院甚至在其铸造的银币上压制Silphium图案，作为帝国繁荣的象征。塞琉古帝国在公元前3世纪初攻占昔兰尼后废止本地铸币，此币发行于城市沦陷后的罗马统治早期，由当地官员以原塞琉古模具或本地模具发行，正面阿波罗·卡内奥斯（Apollo Carneius，羊角神）头像，羊角与桂冠共存，象征城邦保护神的神圣权威；背面Silphium枝叶繁茂，茎粗壮有力，果实心脏形，根系卷曲——这一经典图式在昔兰尼钱币上延续了两百余年。令人唏嘘的是，公元1世纪Silphium已彻底灭绝，原因可能是过度采集、地震破坏与土壤退化三重打击。</t>
+          <t>本都王国（Pontos）位于安纳托利亚北部黑海沿岸，阿米索斯（Amisos，今土耳其萨姆松）是其最重要的港口城市之一。本都王国自米特里达梯一世建立，经历了数代君主的统治。约BC 120年，米特里达梯六世（Mithradates VI Eupator）继位，由于年幼由母亲摄政，此枚铜币即发行于这一时期。丰饶角象征富饶，狄俄斯库里兄弟的双帽子则暗示港口的航海保护，八芒星则代表这对孪生神兄弟。铭文ΑΜΙΣΟΥ即阿米索斯的希腊文拼写。</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T16:08:56</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>a10f3c3</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2794,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2907,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -3123,7 +3130,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -3216,7 +3223,6 @@
           <t>拍卖</t>
         </is>
       </c>
-      <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr">
         <is>
           <t>2024</t>
@@ -3237,11 +3243,9 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
-        </is>
-      </c>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
+          <t>2026-07-07T16:02:53</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3342,7 +3346,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3459,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-07-07T15:40:28</t>
+          <t>2026-07-07T16:02:53</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: GR-002和GK-011 provenance更正; GK-011 obverse改回用户原始描述（珀尔修斯winged bust）
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -2465,7 +2465,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>本都·阿米索斯 米特里达梯六世/丰饶角铜币</t>
+          <t>本都·阿米索斯 珀尔修斯/丰饶角铜币</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>正面: 米特里达梯六世戴王缰带头向右胸像</t>
+          <t>正面: winged and draped bust of Perseus right</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2544,7 +2544,7 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2562,13 +2562,13 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-07T16:08:56</t>
+          <t>2026-07-07T16:17:38</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>a10f3c3</t>
+          <t>bde5659</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
add ROM-007: P.Licinius Nerva投票德纳里乌斯 BC113-112; 修复save_coin.py provenance链条解析（取最后一次出现）
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -2541,7 +2541,6 @@
           <t>Auction Ancients 34</t>
         </is>
       </c>
-      <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr">
         <is>
           <t>2026</t>
@@ -2565,7 +2564,6 @@
           <t>2026-07-07T16:17:38</t>
         </is>
       </c>
-      <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr">
         <is>
           <t>bde5659</t>
@@ -2919,42 +2917,42 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>伦巴第铁王冠</t>
+          <t>Comitium 公民投票场景</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>拿破仑皇帝兼意大利国王1索尔迪铜币</t>
+          <t>罗马共和国 P. 李锡尼亚·内尔瓦 投票德纳里乌斯</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>伦巴第铁王冠 · 米兰造币厂</t>
+          <t>Comitium 公民投票场景 · Crawford 292/1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>AD 1811</t>
+          <t>BC 113-BC 112</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1 Soldo 索尔迪</t>
+          <t>Denarius 德纳里乌斯</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Copper 铜 · 22mm · ~4.6g</t>
+          <t>Silver 银 · 18mm · 3.70g · 轴 9h</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>NGC-AU50</t>
+          <t>Good Very Fine; beautiful old cabinet tone</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Crawford-292/1; BMCRR Italy-526; RSC Licinia-7</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2964,45 +2962,50 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>正面: 拿破仑面向左之桂冠头像 · 铭文 NAPOLEONE IMPERATORE E RE（拿破仑皇帝兼国王）· 底部署名 1811 · 造币厂标记 M（Milano，米兰）</t>
+          <t>正面: 戴头盔的罗马女神（Roma）向左胸像 · 手持盾牌与长矛于肩后 · 头顶上方有新月 · 铭文 ROMA 纵列于后方 · 币值标记位于前方</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>背面: 伦巴第铁王冠（Lombardy Iron Crown）· 顶部铭文 REGNO D'ITALIA（意大利王国）· 底部面值 1 SOLDO</t>
+          <t>背面: 三名公民在 comitium（公民大会广场）投票的场景 · 一名选民从下方助手手中接过选票 · 另一选民将选票投入票箱（cista）· 上方铭文 P·NERVA · 右上方字段有一张标有字母 P 的选票（tabella）</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>拿破仑, 意大利王国, 拿破仑帝国, 索尔迪, 伦巴第铁王冠, 米兰, 19世纪, 1800-1815, NGC, 铜币, 意大利统一运动</t>
+          <t>罗马共和国, P.李锡尼亚·内尔瓦, 德纳里乌斯, 投票场景, 银币, 秘密投票法, Comitium, Lex Gabinia, 李锡尼亚氏族</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>¥992</t>
+          <t>£360</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>CNY</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>992</v>
+        <v>3312</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>云台主人</t>
+          <t>The Coin CABINET</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>私洽</t>
+          <t>Auction Ancients 34</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>295</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -3010,14 +3013,21 @@
           <t>images/ROM-007.jpg</t>
         </is>
       </c>
+      <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr">
         <is>
-          <t>1811年拿破仑帝国鼎盛时期，意大利王国（Regno d'Italia）铸造的1索尔迪铜币。米兰造币厂（Mint Mark M）出品，编号NGC-AU50，成交价992元，来源云台主人2025年10月。 拿破仑于1805年在米兰加冕为意大利国王，随后在意大利领土上推行与法兰西帝国一致的行政、金融与货币体系。意大利王国使用法国货币标准：里拉（Lira）为记账单位，辅币包括索尔迪（Soldo，1里拉=20索尔迪）和分（Centesimo，1索尔迪=5分）。此枚1索尔迪铜币正面为拿破仑桂冠头像，铭文NAPOLEONE IMPERATORE E RE（拿破仑皇帝兼国王），底部署名1811与造币厂标记M（Milano）。背面为伦巴第铁王冠（Lombardy Iron Crown）——意大利统一运动的核心象征，王冠中心铭刻REGNO D'ITALIA（意大利王国），底部面值1 SOLDO。 伦巴第铁王冠（Lombardy Iron Crown）相传以钉死耶稣的圣钉铸造，直径4.5厘米，重约250克，外包金箔，内环为铁质。它是中世纪伦巴第王国及意大利独立运动的重要象征，拿破仑在取得马伦戈战役（1800年）后于伦巴第加冕时使用过此王冠。将铁王冠图案铸于钱币，既是拿破仑宣示其意大利王权的政治行为，也暗示他继承了意大利乃至神圣罗马帝国的历史正统性。此币NGC AU50品相，币面光亮，边齿锐利，是意大利王国拿破仑时期铜币的典型收藏品。</t>
+          <t>这是罗马共和国晚期最著名的投票场景德纳里乌斯之一，由造币三巨头（tresvir monetalis）P. Licinius Nerva 于公元前113-112年铸造。 背面所描叙的公民投票场景是罗马共和政治史中极其罕见的图像记录：一名选民从下方助手手中接过选票（tabella），另一名选民将选票投入票箱（cista），右上方有一张标有字母P的选票。 这一图景与罗马秘密投票制（tabella）的历史性改革密切相关。公元前139年的 Lex Gabinia 引入了立法大会中的无记名投票，公元前137年的 Lex Cassia 将其扩展至司法审判，公元前131年的 Lex Papiria 进一步强化其适用。这一系列改革标志着罗马民主程序的重要进化——公民不再需要公开自己的投票立场。 选票上的P字学界通常解释为某位候选人姓名的首字母缩写，具体指代仍有争议。 P. Licinius Nerva 出身李锡尼亚氏族（gens Licinia），其本身日后也成为罗马政坛重要人物。</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-07-06T17:43:24</t>
+          <t>2026-07-07T16:33:53</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>a90e8d4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ROM-008: update C. Cassius Longinus denarius - correct ref to Crawford 413/1; add weight/diameter/die axis/provenance/price; obverse diadem added from user text
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z27"/>
+  <dimension ref="A1:Z28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -657,12 +657,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Auctionaes AG</t>
+          <t>Numismatik Naumann</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Auction 7</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>1977</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:52</t>
+          <t>2026-07-07T17:23:16</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Camerarius Numizmatika</t>
+          <t>Solidus Numismatik</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>NGC</t>
+          <t>Numismatik Naumann</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:18</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -2561,12 +2561,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-07T16:17:38</t>
-        </is>
-      </c>
-      <c r="Z19" t="inlineStr">
-        <is>
-          <t>bde5659</t>
+          <t>2026-07-07T17:23:18</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2787,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:18</t>
         </is>
       </c>
     </row>
@@ -2905,7 +2900,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:18</t>
         </is>
       </c>
     </row>
@@ -2962,12 +2957,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>正面: 戴头盔的罗马女神（Roma）向左胸像 · 手持盾牌与长矛于肩后 · 头顶上方有新月 · 铭文 ROMA 纵列于后方 · 币值标记位于前方</t>
+          <t>正面: 戴头盔的罗马女神（Roma）左侧胸像，手持盾牌，长矛扛于肩后。</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>背面: 三名公民在 comitium（公民大会广场）投票的场景 · 一名选民从下方助手手中接过选票 · 另一选民将选票投入票箱（cista）· 上方铭文 P·NERVA · 右上方字段有一张标有字母 P 的选票（tabella）</t>
+          <t>背面: X / P·NERVA，两名公民在公民大会广场（comitium）投票，左侧公民手持选票板（tabella），右侧公民将选票投入开启的投票箱（cista）。底部横线装饰（a line of dots）。</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3013,7 +3008,9 @@
           <t>images/ROM-007.jpg</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr"/>
+      <c r="V23" t="n">
+        <v>258334</v>
+      </c>
       <c r="W23" t="inlineStr">
         <is>
           <t>这是罗马共和国晚期最著名的投票场景德纳里乌斯之一，由造币三巨头（tresvir monetalis）P. Licinius Nerva 于公元前113-112年铸造。 背面所描叙的公民投票场景是罗马共和政治史中极其罕见的图像记录：一名选民从下方助手手中接过选票（tabella），另一名选民将选票投入票箱（cista），右上方有一张标有字母P的选票。 这一图景与罗马秘密投票制（tabella）的历史性改革密切相关。公元前139年的 Lex Gabinia 引入了立法大会中的无记名投票，公元前137年的 Lex Cassia 将其扩展至司法审判，公元前131年的 Lex Papiria 进一步强化其适用。这一系列改革标志着罗马民主程序的重要进化——公民不再需要公开自己的投票立场。 选票上的P字学界通常解释为某位候选人姓名的首字母缩写，具体指代仍有争议。 P. Licinius Nerva 出身李锡尼亚氏族（gens Licinia），其本身日后也成为罗马政坛重要人物。</t>
@@ -3021,13 +3018,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-07-07T16:33:53</t>
-        </is>
-      </c>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr">
-        <is>
-          <t>a90e8d4</t>
+          <t>2026-07-07T17:23:18</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3131,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:18</t>
         </is>
       </c>
     </row>
@@ -3225,17 +3216,17 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Classical Numismatic Group</t>
+          <t>The Coin CABINET</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>拍卖</t>
+          <t>Auction Ancients 34</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3253,7 +3244,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:18</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3347,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
+          <t>2026-07-07T17:23:17</t>
         </is>
       </c>
     </row>
@@ -3469,9 +3460,121 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-07-07T16:02:53</t>
-        </is>
-      </c>
+          <t>2026-07-07T17:23:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ROM-008</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Vesta</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Vesta · Rome Mint · 63 BC</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>63 BC</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Denarius 德纳里乌斯</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Silver 银 · 20mm · 3.70g · 轴 6h</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>EF</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Crawford 413/1; BMCRR Rome 3936; RSC Cassia 10</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>roman</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>正面: Veiled and diademed bust of Vesta left, holding libation cup (kylix); control mark before face.</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>背面: Voter standing left, placing tablet marked 'V' into cista (ballot box); LONGIN · III · V to right; three lines in exergue; control mark in field.</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>罗马共和国, C.卡西乌斯·朗基努斯, 德纳里乌斯, 维斯塔, 秘密投票, Crawford 413</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>£360</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>3312</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>The Coin CABINET</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Auction Ancients 34</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>images/ROM-008.jpg</t>
+        </is>
+      </c>
+      <c r="V28" t="n">
+        <v>311292</v>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>此币正面图案献给 L. Cassius Longinus Ravilla——这位 L. Cassius Longinus（造币官）的祖父，他是一位备受尊敬的裁判官和法学家。公元前 113 年，Ravilla 主持了对三名维斯塔处女（Vestal Virgin）的审判，指控她们破坏贞操，最终判定其中两人有罪并处以死刑——这一事件在罗马历史上极为罕见，体现了罗马司法的严厉一面。他的银币背面所描绘的，正是他担任保民官期间（公元前 137 年）引入的罗马秘密投票制度的运作场景。这一制度革新标志着罗马公民无需在公开场合表明投票立场——投票权的引入深刻影响了罗马的民主进程。</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>2026-07-07T17:23:18</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add GR-004: Chersonesos Taurica lion forepart 1/2 drachm, BC 4th c., ¥1,208
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z28"/>
+  <dimension ref="A1:Z29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2573,67 +2573,67 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SELEUCID EMPIRE</t>
+          <t>Ionia, Miletos</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>塞琉古帝国塞琉古一世铜币</t>
+          <t>米利都·阿尔康 1德拉克马银币</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>SELEUCID EMPIRE · ELEPHANT &amp; BUCERAS</t>
+          <t>Ionia, Miletos · Alkon</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>公元前312-前281年</t>
+          <t>BC 260-250</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Chalkous 铜币</t>
+          <t>AR Drachm</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Bronze 青铜 · 22mm · 6.42g</t>
+          <t>Silver · 20mm · 5.29g</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>VF</t>
+          <t>GVF</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Deppert-Lippitz 515; SNG von Aulock -; SNG Copenhagen -; BMC 94</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>greek</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>正面: 亚洲象向右行走 · 体态健壮 · 背上驮有辎重</t>
+          <t>正面: Laureate head of Apollo left</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>背面: 戴牛角之马头向右 · 下方船锚 ⚓ · 铭文 ΒΑΣΙΛΕΩΣ ΣΕΛΕΥΚΟΥ</t>
+          <t>反面: Lion standing to left, looking back at star with eight rays; monogram over T before, ΑΛΚΩΝ in exergue</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>塞琉古, 塞琉古一世, 胜利者, Nikator, 亚洲象, 布克法罗斯, Bucephalus, 阿帕美亚, 伊普苏斯, 继业者战争, 船锚</t>
+          <t>GK, 米利都, 阿波罗, 狮子, 阿尔康</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>¥360</t>
+          <t>¥3,780</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2642,21 +2642,21 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>360</v>
+        <v>3780</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>西西里晚祷</t>
+          <t>琋语集藏</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>私洽</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2665,16 +2665,21 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>175619</v>
+        <v>2600529</v>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>公元前323年亚历山大大帝骤然离世，其帝国随即陷入继业者战争（War of the Diadochi）。塞琉古（Seleucus）作为亚历山大的近身护卫官，于公元前321年被迫流亡埃及。公元前312年，在托勒密一世的支持下，塞琉古重返巴比伦，宣布独立，开启了塞琉古帝国长达两百余年的统治，是年便成为塞琉古纪元的元年。公元前301年伊普苏斯战役（Battle of Ipsus），塞琉古与利西马科斯（Lysimachus）联手击败安提柯（Antigonus），瓜分亚历山大帝国的东部版图，塞琉古一跃成为从安纳托利亚延伸至印度的庞大帝国之君，领土面积仅次于孔雀王朝印度。 阿帕美亚（Apamaea on the Orontes）位于奥隆特斯河畔，是塞琉古帝国最繁华的城市之一，以其母——塞琉古一世之妻阿帕美亚（Apama）命名，与安条克、塞琉西亚并列为帝国三大都城。 此币正面亚洲象向右行走，象征塞琉古从印度孔雀王朝君主旃陀罗笈多（Chandragupta）手中换取的五百头战象，这些战象是伊普苏斯战役决定性胜利的关键；背面戴牛角之马头为布克法罗斯（Bucephalus）的形象，据传是亚历山大大帝的传奇坐骑，塞琉古以布克法罗斯自比，昭示其作为亚历山大正统继承人的身份；船锚则暗指塞琉古大腿根部形似锚状的胎记，同时也象征其祖先尼卡托尔（Nicator，意为「胜利者」）作为亚历山大海军指挥官与腓力二世时期的海军将领之出身，将希腊世界的海上传统与新帝国紧紧相连。</t>
+          <t>这枚币来自古希腊首位哲学家泰勒斯的家乡米利都。泰勒斯是古希腊七贤之一，西方思想史上第一个有记载有名字留下来的思想家，被称为"科学和哲学之祖"。据希罗多德记载，泰勒斯曾准确预言了一次日食（学界推测为公元前585年5月28日），并提出"水是万物本源"的命题。米利都位于爱奥尼亚海岸，是公元前7至5世纪爱琴海世界最繁盛的工商业城邦之一，殖民范围远及埃及与黑海沿岸，由铸币官阿尔康（ΑΛΚΩΝ）发行此币。</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-07T14:57:53</t>
+          <t>2026-07-07T17:45:09</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>b3a8a12</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3480,6 @@
           <t>Vesta</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>Vesta · Rome Mint · 63 BC</t>
@@ -3549,7 +3553,6 @@
           <t>Auction Ancients 34</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr">
         <is>
           <t>2026</t>
@@ -3573,8 +3576,126 @@
           <t>2026-07-07T17:23:18</t>
         </is>
       </c>
-      <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>GR-004</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>CHERSONESOS TAURICA</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>切尔森尼索斯 狮子半德银币</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CHERSONESOS TAURICA · 4th Century BC</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>BC 4th century 公元前4世纪</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1/2 Drachm 半德拉克马</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Silver 银 · 12.9mm · 2.39g</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>greek</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>正面: forepart of lion looking back 狮子半身像回望</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>背面: 四格戳记 quadripartite incuse square with symbols</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>黑海, 切尔森尼索斯, 陶里卡, 狮子, 米利都殖民, 公元前4世纪</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>¥1,208</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>1208</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>琋语集藏</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>images/GR-004.jpg</t>
+        </is>
+      </c>
+      <c r="V29" t="n">
+        <v>2197827</v>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>切尔森尼索斯（Chersonesos Taurica）是位于黑海北岸（现代克里米亚半岛）的重要希腊殖民城邦，约公元前5世纪由米利都（Miletus）殖民者建立。该城邦控制着黑海北岸的贸易航线，是古代世界重要的粮食和奴隶贸易中心。公元前438年，切尔森尼索斯加入雅典主导的提洛同盟（Athenian Delian League），在伯罗奔尼撒战争期间扮演重要角色。&lt;br&gt;&lt;br&gt;正面描绘的狮子形象（lion forepart）是黑海希腊殖民城市标志性的造币题材，象征着力量与城邦的军事实力。回望姿态的狮子在古典希腊艺术中极为罕见，增加了这枚币的艺术价值和特殊性。背面四格戳记（quadripartite incuse square）是古典时期希腊银币的标准特征，每个格子内的小符号（字母或谷穗）是造币官或城邦徽记，反映了城邦的内部行政体系。</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>2026-07-07T17:52:10</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>0555589</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
新增 NI-003 意大利王国 3 Centesimi 1813 米兰铜币
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="钱币目录" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="钱币目录" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z29"/>
+  <dimension ref="A1:Z33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -685,12 +685,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Deinomenid 四兄弟（Gelon、Hieron、Thrasybulus、Polyzelus）于 BC 485 年建立僭主统治，Syracuse 由此跃升为西地中海最强希腊城邦。BC 480 年希梅拉战役（Himera）—— Gelon 联合 Akragas 城大败迦太基，古典作家希罗多德将其与同年的萨拉米斯海战并列为希腊人东西方战略的标志性胜利。四马战车（Quadriga）向右疾驰、Nike 飞降加冕，直接象征此类军事胜利与神圣赐福。背面 Arethusa 头像被四只海豚环绕——海豚是 Syracuse 延续数百年的城徽，寓意城市被海洋拥抱的地理与文化双重身份。此币属 Boehringer 115 标准版式，代表古典西西里艺术巅峰的前夜。</t>
+          <t>Deinomenid 四兄弟(Gelon、Hieron、Thrasybulus、Polyzelus)于 BC 485 年建立僭主统治,Syracuse 由此跃升为西地中海最强希腊城邦。BC 480 年希梅拉战役(Himera)-- Gelon 联合 Akragas 城大败迦太基,古典作家希罗多德将其与同年的萨拉米斯海战并列为希腊人东西方战略的标志性胜利。四马战车(Quadriga)向右疾驰、Nike 飞降加冕,直接象征此类军事胜利与神圣赐福。背面 Arethusa 头像被四只海豚环绕--海豚是 Syracuse 延续数百年的城徽,寓意城市被海洋拥抱的地理与文化双重身份。此币属 Boehringer 115 标准版式,代表古典西西里艺术巅峰的前夜。</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:16</t>
+          <t>2026-07-12T13:55:55</t>
         </is>
       </c>
     </row>
@@ -798,12 +798,12 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>亚历山大造币厂是罗马帝国内最特殊的货币发行地——奥古斯都征服托勒密埃及后，刻意保留其希腊化造币传统，以希腊铭文和神祇为主图，与拉丁传统形成鲜明对比。从提比略起，行省埃及币每位皇帝均有铸造，且每年更换纪年版式。此枚为尼禄第14年（L IΔ = RY 14 = AD 67/68），对应其希腊巡游期间。尼禄辐射冠头像左向，强调皇帝与太阳神的联系——尼禄晚年尤其致力建构「太阳神」身份。肩披 Aegis 原为雅典娜护胸甲，被罗马皇帝借用以象征神佑（divine protection）。背面天后赫拉（Hera）戴冠披巾头像右向，延续希腊化时代亚历山大对城市守护神的崇拜传统。</t>
+          <t>亚历山大造币厂是罗马帝国内最特殊的货币发行地--奥古斯都征服托勒密埃及后,刻意保留其希腊化造币传统,以希腊铭文和神祇为主图,与拉丁传统形成鲜明对比。从提比略起,行省埃及币每位皇帝均有铸造,且每年更换纪年版式。此枚为尼禄第14年(L IΔ = RY 14 = AD 67/68),对应其希腊巡游期间。尼禄辐射冠头像左向,强调皇帝与太阳神的联系--尼禄晚年尤其致力建构「太阳神」身份。肩披 Aegis 原为雅典娜护胸甲,被罗马皇帝借用以象征神佑(divine protection)。背面天后赫拉(Hera)戴冠披巾头像右向,延续希腊化时代亚历山大对城市守护神的崇拜传统。</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:55</t>
         </is>
       </c>
     </row>
@@ -860,12 +860,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>正面: ΑΛΕΞΑΝΔΡΟΥ · 亚历山大大帝戴阿蒙（Ammon）角状头饰头像右</t>
+          <t>正面: ΑΛΕΞΑΝΔΡΟΥ · 亚历山大大帝戴阿蒙(Ammon)角状头饰头像右</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>背面: ΑΘΗΝΑ · 雅典娜戴盔持盾矛立像右 · ΒΑΣΙΛΕΩΣ ΛΥΣΙΜΑΧΟΥ · ΑΘΗΝΑΣ（造币厂控制标记）</t>
+          <t>背面: ΑΘΗΝΑ · 雅典娜戴盔持盾矛立像右 · ΒΑΣΙΛΕΩΣ ΛΥΣΙΜΑΧΟΥ · ΑΘΗΝΑΣ(造币厂控制标记)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -901,12 +901,12 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>吕西马科斯（Lysimachos，BC 360-281）是亚历山大大帝的六位近身侍卫（Somatophylax）之一，于BC 306/305年在色雷斯自立为王，建都莱普提昂杜斯（Lysimotelia），随后在其治下的色雷斯及小亚细亚地区大规模铸造四德拉克马金币。Lampsakos（兰普萨科斯）位于达达尼尔海峡入口，是吕西马科斯王国最重要的造币中心之一，掌控着从本都-潘提卡彭至爱琴海的贵金属流通命脉。&lt;br&gt;&lt;br&gt;吕西马科斯四德拉克马正面沿用经典的亚历山大阿蒙之角（Ammon Horn）形象——这一肖像自BC 336年起便随亚历山大的军事扩张流通于整个希腊化世界，是最早、最具辨识度的希腊化君主肖像。亚历山大通过宣称自己是埃及阿蒙神之子（Jupiter Ammon）来建构其神性血统，吕西马科斯沿用这一肖像，既是政治宣传，也是对亚历山大开创的希腊化君主制iconography（肖像体系）的直接继承。&lt;br&gt;&lt;br&gt;背面雅典娜·阿尔基德莫斯（Athena Alkidemos）是马其顿及亚历山大继承者们偏爱的战神形象——手持阿尔基（Alche，阿克顿的神盾）和矛，身披盔甲配狮皮头盔。Lampsakos造币厂以ΑΘΗΝΑΣ作为控制标记（control mark），用于区分不同批次和工匠。吕西马科斯四德拉克马是希腊化时期发行量最大、流通最广的硬币版式之一。</t>
+          <t>吕西马科斯(Lysimachos,BC 360-281)是亚历山大大帝的六位近身侍卫(Somatophylax)之一,于BC 306/305年在色雷斯自立为王,建都莱普提昂杜斯(Lysimotelia),随后在其治下的色雷斯及小亚细亚地区大规模铸造四德拉克马金币。Lampsakos(兰普萨科斯)位于达达尼尔海峡入口,是吕西马科斯王国最重要的造币中心之一,掌控着从本都-潘提卡彭至爱琴海的贵金属流通命脉。&lt;br&gt;&lt;br&gt;吕西马科斯四德拉克马正面沿用经典的亚历山大阿蒙之角(Ammon Horn)形象--这一肖像自BC 336年起便随亚历山大的军事扩张流通于整个希腊化世界,是最早、最具辨识度的希腊化君主肖像。亚历山大通过宣称自己是埃及阿蒙神之子(Jupiter Ammon)来建构其神性血统,吕西马科斯沿用这一肖像,既是政治宣传,也是对亚历山大开创的希腊化君主制iconography(肖像体系)的直接继承。&lt;br&gt;&lt;br&gt;背面雅典娜·阿尔基德莫斯(Athena Alkidemos)是马其顿及亚历山大继承者们偏爱的战神形象--手持阿尔基(Alche,阿克顿的神盾)和矛,身披盔甲配狮皮头盔。Lampsakos造币厂以ΑΘΗΝΑΣ作为控制标记(control mark),用于区分不同批次和工匠。吕西马科斯四德拉克马是希腊化时期发行量最大、流通最广的硬币版式之一。</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -963,12 +963,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>正面: NEPΩ KΛAV KAIΣ ΣEB ΓEP AV · 尼禄头戴光芒冠左向胸像，佩戴Aegis；L IΔ</t>
+          <t>正面: NEPΩ KΛAV KAIΣ ΣEB ΓEP AV · 尼禄头戴光芒冠左向胸像,佩戴Aegis;L IΔ</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>背面: AKTIOΣ AΠOΛΛΩN · 阿波罗右向胸像，肩扛箭袋；星形标记</t>
+          <t>背面: AKTIOΣ AΠOΛΛΩN · 阿波罗右向胸像,肩扛箭袋;星形标记</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1014,12 +1014,12 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>罗马行省埃及是帝国内唯一被奥古斯都禁止铸造"皇帝肖像"和"拉丁铭文"的行省——奥古斯都征服托勒密埃及后，刻意保留当地希腊传统以安抚亚历山大里亚民众。亚历山大造币厂沿袭希腊化传统，以希腊铭文和神祇为主图，且&lt;b&gt;每年更换版式&lt;/b&gt;。年份标记 L IΔ 采用"奥古斯都纪年+皇帝在位年"双轨制，即奥古斯都纪年 14 + 尼禄 RY 14 = 公元 67/68 年。 背面 AKTIOΣ AΠOΛΛΩN（阿克提乌斯·阿波罗）是奥古斯都纪念公元前 31 年阿克提乌姆海战击败安东尼与克娄巴特拉的神祇。尼禄 RY 14（67 AD）正值其希腊巡游期间、宣布"希腊自由"的同一年，埃及币上仍延续这一图式，反映出罗马对行省货币传统的政治延续性。 关于"BI"：Billon 是含银量仅约 18–25% 的银铜合金。罗马政府有意降低埃及币成色以遏制贵金属外流——罗马本土的"银币"（denarius）含银量约 80%，而埃及四德拉克马只值其 1/3 不到。这使行省埃及币成为研究罗马经济分层的独特样本。</t>
+          <t>罗马行省埃及是帝国内唯一被奥古斯都禁止铸造"皇帝肖像"和"拉丁铭文"的行省--奥古斯都征服托勒密埃及后,刻意保留当地希腊传统以安抚亚历山大里亚民众。亚历山大造币厂沿袭希腊化传统,以希腊铭文和神祇为主图,且&lt;b&gt;每年更换版式&lt;/b&gt;。年份标记 L IΔ 采用"奥古斯都纪年+皇帝在位年"双轨制,即奥古斯都纪年 14 + 尼禄 RY 14 = 公元 67/68 年。 背面 AKTIOΣ AΠOΛΛΩN(阿克提乌斯·阿波罗)是奥古斯都纪念公元前 31 年阿克提乌姆海战击败安东尼与克娄巴特拉的神祇。尼禄 RY 14(67 AD)正值其希腊巡游期间、宣布"希腊自由"的同一年,埃及币上仍延续这一图式,反映出罗马对行省货币传统的政治延续性。 关于"BI":Billon 是含银量仅约 18-25% 的银铜合金。罗马政府有意降低埃及币成色以遏制贵金属外流--罗马本土的"银币"(denarius)含银量约 80%,而埃及四德拉克马只值其 1/3 不到。这使行省埃及币成为研究罗马经济分层的独特样本。</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>安东尼·庇护 塞斯特提乌斯（LIBERTAS COS IIII）</t>
+          <t>安东尼·庇护 塞斯特提乌斯(LIBERTAS COS IIII)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AD 145-161（TR P XVIII = AD 155/6）</t>
+          <t>AD 145-161(TR P XVIII = AD 155/6)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>背面: LIBERTAS COS IIII / S - C · 自由女神左站，持 pileus + vindicta</t>
+          <t>背面: LIBERTAS COS IIII / S - C · 自由女神左站,持 pileus + vindicta</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1127,12 +1127,12 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>安东尼·庇护（Antoninus Pius，138-161 AD）是罗马帝国"五贤帝"的第四位，以和平、不扩张、重法律著称。此币发行于其统治晚期（TR P XVIII = AD 155/6），距罗马大火已约 11 年（64 AD 尼禄时期），距哈德良长城建成约 20 年（约 142 AD）。 &lt;b&gt;LIBERTAS&lt;/b&gt;（自由女神）是五贤帝时期反复出现的主题：自由女神站立，左手持自由帽（&lt;b&gt;pileus&lt;/b&gt;），右手持"vindicta"（&lt;b&gt;liberty rod 自由权杖&lt;/b&gt;）。这个组合源自罗马解放奴隶仪式（manumissio）：主人用权杖触奴隶头，宣布"hunc hominem liberum esse volo"（我愿此人自由），奴隶戴上自由帽。 五贤帝刻意铸造 LIBERTAS 主题，意在强调&lt;b&gt;元老院与皇帝共治&lt;/b&gt;的"共和表象"——虽然实行帝制，但理论上"罗马公民自由"仍在。安东尼·庇护尤其重视此意象，因为其继位未经内战，强调"合法继承"与"恢复自由"是政治需要。 背面铭文 &lt;b&gt;LIBERTAS COS IIII&lt;/b&gt; 中 COS IIII = 第四次执政官（约 AD 145），S-C 分别立于左右（Senatus Consulto = 元老院决议）。</t>
+          <t>安东尼·庇护(Antoninus Pius,138-161 AD)是罗马帝国"五贤帝"的第四位,以和平、不扩张、重法律著称。此币发行于其统治晚期(TR P XVIII = AD 155/6),距罗马大火已约 11 年(64 AD 尼禄时期),距哈德良长城建成约 20 年(约 142 AD)。 &lt;b&gt;LIBERTAS&lt;/b&gt;(自由女神)是五贤帝时期反复出现的主题:自由女神站立,左手持自由帽(&lt;b&gt;pileus&lt;/b&gt;),右手持"vindicta"(&lt;b&gt;liberty rod 自由权杖&lt;/b&gt;)。这个组合源自罗马解放奴隶仪式(manumissio):主人用权杖触奴隶头,宣布"hunc hominem liberum esse volo"(我愿此人自由),奴隶戴上自由帽。 五贤帝刻意铸造 LIBERTAS 主题,意在强调&lt;b&gt;元老院与皇帝共治&lt;/b&gt;的"共和表象"--虽然实行帝制,但理论上"罗马公民自由"仍在。安东尼·庇护尤其重视此意象,因为其继位未经内战,强调"合法继承"与"恢复自由"是政治需要。 背面铭文 &lt;b&gt;LIBERTAS COS IIII&lt;/b&gt; 中 COS IIII = 第四次执政官(约 AD 145),S-C 分别立于左右(Senatus Consulto = 元老院决议)。</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>埃及·尼禄等亚历山大四德拉克马（批量×9）</t>
+          <t>埃及·尼禄等亚历山大四德拉克马(批量×9)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>54–68+ AD（多位皇帝）</t>
+          <t>54-68+ AD(多位皇帝)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>正面: 多位皇帝头像（Nero为主，含Claudius等）</t>
+          <t>正面: 多位皇帝头像(Nero为主,含Claudius等)</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1240,12 +1240,12 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>Numismatik Naumann Auction 154 批量Lot，包含9枚亚历山大造币厂Billon Tetradrachm，主要涵盖尼禄时期及同时代其他皇帝。正面多位皇帝肖像（含NEPΩN KΛAY KAIΣ ΣEB ΓEP等多版式），背面鹰立持权杖、L年份标记等典型亚历山大类型。部分带Aegis争议细节。</t>
+          <t>Numismatik Naumann Auction 154 批量Lot,包含9枚亚历山大造币厂Billon Tetradrachm,主要涵盖尼禄时期及同时代其他皇帝。正面多位皇帝肖像(含NEPΩN KΛAY KAIΣ ΣEB ΓEP等多版式),背面鹰立持权杖、L年份标记等典型亚历山大类型。部分带Aegis争议细节。</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -1302,12 +1302,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>正面: 宙斯月桂冠头像右向（古典肖像艺术巅峰）</t>
+          <t>正面: 宙斯月桂冠头像右向(古典肖像艺术巅峰)</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>背面: ΦΙΛΙΠΠΟΥ · 持棕榈少年骑骏马右行·下双控：海豚 + pellet-in-Π</t>
+          <t>背面: ΦΙΛΙΠΠΟΥ · 持棕榈少年骑骏马右行·下双控:海豚 + pellet-in-Π</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1353,12 +1353,12 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>亚历山大大帝之父腓力二世——马其顿王国奠基者，公元前338年喀罗尼亚战役确立希腊霸权。&lt;strong&gt;安菲波利斯造币厂&lt;/strong&gt;是其在位期间最重要的铸币中心，币面宙斯月桂冠头像为古希腊钱币肖像艺术巅峰。背面青年骑手&lt;strong&gt;手持棕榈枝&lt;/strong&gt;纪念腓力公元前356年奥运会马赛冠军——当届马其顿首次参赛即夺金，是其政治生涯的重要象征。马下双控制标记（controls）：&lt;strong&gt;海豚&lt;/strong&gt;（ΔΕΛΦΙΣ delphis）= 安菲波利斯海港城市标志，&lt;strong&gt;pellet-in-Π&lt;/strong&gt; = 特定年版或印模组的官方标识。Le Rider pl. 46, 19 将此版式归入腓力二世"Group C"晚期安菲波利斯币。NGC 6636427-001 认证，GVF 品相。</t>
+          <t>亚历山大大帝之父腓力二世--马其顿王国奠基者,公元前338年喀罗尼亚战役确立希腊霸权。&lt;strong&gt;安菲波利斯造币厂&lt;/strong&gt;是其在位期间最重要的铸币中心,币面宙斯月桂冠头像为古希腊钱币肖像艺术巅峰。背面青年骑手&lt;strong&gt;手持棕榈枝&lt;/strong&gt;纪念腓力公元前356年奥运会马赛冠军--当届马其顿首次参赛即夺金,是其政治生涯的重要象征。马下双控制标记(controls):&lt;strong&gt;海豚&lt;/strong&gt;(ΔΕΛΦΙΣ delphis)= 安菲波利斯海港城市标志,&lt;strong&gt;pellet-in-Π&lt;/strong&gt; = 特定年版或印模组的官方标识。Le Rider pl. 46, 19 将此版式归入腓力二世"Group C"晚期安菲波利斯币。NGC 6636427-001 认证,GVF 品相。</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1466,12 +1466,12 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>公元前323年亚历山大大帝骤然离世，其帝国随即陷入继业者战争（War of the Diadochi）。塞琉古（Seleucus）作为亚历山大的近身护卫官，于公元前321年被迫流亡埃及。公元前312年，在托勒密一世的支持下，塞琉古重返巴比伦，宣布独立，开启了塞琉古帝国长达两百余年的统治，是年便成为塞琉古纪元的元年。公元前301年伊普苏斯战役（Battle of Ipsus），塞琉古与利西马科斯（Lysimachus）联手击败安提柯（Antigonus），瓜分亚历山大帝国的东部版图，塞琉古一跃成为从安纳托利亚延伸至印度的庞大帝国之君，领土面积仅次于孔雀王朝印度。 阿帕美亚（Apamaea on the Orontes）位于奥隆特斯河畔，是塞琉古帝国最繁华的城市之一，以其母——塞琉古一世之妻阿帕美亚（Apama）命名，与安条克、塞琉西亚并列为帝国三大都城。 此币正面亚洲象向右行走，象征塞琉古从印度孔雀王朝君主旃陀罗笈多（Chandragupta）手中换取的五百头战象，这些战象是伊普苏斯战役决定性胜利的关键；背面戴牛角之马头为布克法罗斯（Bucephalus）的形象，据传是亚历山大大帝的传奇坐骑，塞琉古以布克法罗斯自比，昭示其作为亚历山大正统继承人的身份；船锚则暗指塞琉古大腿根部形似锚状的胎记，同时也象征其祖先尼卡托尔（Nicator，意为「胜利者」）作为亚历山大海军指挥官与腓力二世时期的海军将领之出身，将希腊世界的海上传统与新帝国紧紧相连。</t>
+          <t>公元前323年亚历山大大帝骤然离世,其帝国随即陷入继业者战争(War of the Diadochi)。塞琉古(Seleucus)作为亚历山大的近身护卫官,于公元前321年被迫流亡埃及。公元前312年,在托勒密一世的支持下,塞琉古重返巴比伦,宣布独立,开启了塞琉古帝国长达两百余年的统治,是年便成为塞琉古纪元的元年。公元前301年伊普苏斯战役(Battle of Ipsus),塞琉古与利西马科斯(Lysimachus)联手击败安提柯(Antigonus),瓜分亚历山大帝国的东部版图,塞琉古一跃成为从安纳托利亚延伸至印度的庞大帝国之君,领土面积仅次于孔雀王朝印度。 阿帕美亚(Apamaea on the Orontes)位于奥隆特斯河畔,是塞琉古帝国最繁华的城市之一,以其母--塞琉古一世之妻阿帕美亚(Apama)命名,与安条克、塞琉西亚并列为帝国三大都城。 此币正面亚洲象向右行走,象征塞琉古从印度孔雀王朝君主旃陀罗笈多(Chandragupta)手中换取的五百头战象,这些战象是伊普苏斯战役决定性胜利的关键;背面戴牛角之马头为布克法罗斯(Bucephalus)的形象,据传是亚历山大大帝的传奇坐骑,塞琉古以布克法罗斯自比,昭示其作为亚历山大正统继承人的身份;船锚则暗指塞琉古大腿根部形似锚状的胎记,同时也象征其祖先尼卡托尔(Nicator,意为「胜利者」)作为亚历山大海军指挥官与腓力二世时期的海军将领之出身,将希腊世界的海上传统与新帝国紧紧相连。</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:18</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -1513,12 +1513,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1574,12 +1574,12 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>腓力二世（Philip II）是马其顿王国国王（公元前359-336年），亚历山大大帝之父。他通过军事改革（"马其顿方阵"战术创新）和外交手段，将马其顿从希腊边缘小国提升为希腊霸主，为亚历山大的帝国奠定基础。公元前338年喀罗尼亚战役击败希腊城邦联军后，腓力被尊为希腊世界实际统治者。&lt;br&gt;&lt;br&gt;腓力二世青铜币正面为阿波罗戴王冠头像，阿波罗是希腊神话中的太阳神和音乐之神，也是马其顿王室的重要保护神。背面为青年骑手图像，是马其顿王室标志性的 iconography，铭文"ΦΙΛΙΠΠΟΥ"（腓力普斯/腓力）标明发行者身份。这类青铜小币主要作为辅币流通，用于日常小额交易。</t>
+          <t>腓力二世(Philip II)是马其顿王国国王(公元前359-336年),亚历山大大帝之父。他通过军事改革("马其顿方阵"战术创新)和外交手段,将马其顿从希腊边缘小国提升为希腊霸主,为亚历山大的帝国奠定基础。公元前338年喀罗尼亚战役击败希腊城邦联军后,腓力被尊为希腊世界实际统治者。&lt;br&gt;&lt;br&gt;腓力二世青铜币正面为阿波罗戴王冠头像,阿波罗是希腊神话中的太阳神和音乐之神,也是马其顿王室的重要保护神。背面为青年骑手图像,是马其顿王室标志性的 iconography,铭文"ΦΙΛΙΠΠΟΥ"(腓力普斯/腓力)标明发行者身份。这类青铜小币主要作为辅币流通,用于日常小额交易。</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -1621,12 +1621,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1687,12 +1687,12 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>雅典猫头鹰银币是古希腊最具代表性的货币，从公元前5世纪延续至公元前1世纪，成为古代地中海世界的硬通货。古典时期结束后，雅典于公元前2世纪摆脱马其顿控制，重启银币铸造，采用全新设计风格——新式猫头鹰（New Style）。与古典版相比，新式猫头鹰正面雅典娜头像更为精致，头戴装饰丰富的阿提卡式头盔；背面猫头鹰立于双耳陶罐（amphora）之上，周边环绕橄榄枝，并刻有地方官姓名与徽记，体现了希腊化时期雅典城邦的自治与繁荣。</t>
+          <t>雅典猫头鹰银币是古希腊最具代表性的货币,从公元前5世纪延续至公元前1世纪,成为古代地中海世界的硬通货。古典时期结束后,雅典于公元前2世纪摆脱马其顿控制,重启银币铸造,采用全新设计风格--新式猫头鹰(New Style)。与古典版相比,新式猫头鹰正面雅典娜头像更为精致,头戴装饰丰富的阿提卡式头盔;背面猫头鹰立于双耳陶罐(amphora)之上,周边环绕橄榄枝,并刻有地方官姓名与徽记,体现了希腊化时期雅典城邦的自治与繁荣。</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -1714,12 +1714,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>THRACE · Maroneia (ca. BC 189/8–49/5)</t>
+          <t>THRACE · Maroneia (ca. BC 189/8-49/5)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>ca. BC 189/8–49/5</t>
+          <t>ca. BC 189/8-49/5</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1734,12 +1734,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1795,12 +1795,12 @@
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>马罗尼亚（Maroneia）是色雷斯地区重要的希腊城邦，位于今希腊东北部爱琴海沿岸。该城邦以发达的葡萄酒产业著称，据古希腊作家记载，马罗尼亚的葡萄酒是希腊世界最负盛名的佳酿之一。&lt;br&gt;&lt;br&gt;马罗尼亚四德拉克马正面为年轻酒神狄俄尼索斯（Dionysos）头像，头戴常春藤花冠，额前有装饰带。狄俄尼索斯是古希腊神话中的酒神与戏剧之神，与马罗尼亚的葡萄酒文化紧密相连。背面为裸身站立的狄俄尼索斯，手持葡萄串和两根纳特赫权杖（narthex），身侧有两个组合字母（monogram）作为造币厂或官员标记。铭文"ΔΙΟΝΥΣΟΥ ΣΩΤΗΡΟΣ"意为"狄俄尼索斯，救主"，"ΜΑΡΩΝΙΤΩΝ"意为"马罗尼亚人的"，表明城邦发行身份。</t>
+          <t>马罗尼亚(Maroneia)是色雷斯地区重要的希腊城邦,位于今希腊东北部爱琴海沿岸。该城邦以发达的葡萄酒产业著称,据古希腊作家记载,马罗尼亚的葡萄酒是希腊世界最负盛名的佳酿之一。&lt;br&gt;&lt;br&gt;马罗尼亚四德拉克马正面为年轻酒神狄俄尼索斯(Dionysos)头像,头戴常春藤花冠,额前有装饰带。狄俄尼索斯是古希腊神话中的酒神与戏剧之神,与马罗尼亚的葡萄酒文化紧密相连。背面为裸身站立的狄俄尼索斯,手持葡萄串和两根纳特赫权杖(narthex),身侧有两个组合字母(monogram)作为造币厂或官员标记。铭文"ΔΙΟΝΥΣΟΥ ΣΩΤΗΡΟΣ"意为"狄俄尼索斯,救主","ΜΑΡΩΝΙΤΩΝ"意为"马罗尼亚人的",表明城邦发行身份。</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>背面: 圣乔治策马刺剑，斗篷飞扬，长矛刺杀毒龙，骏马前蹄腾空；龙蜷于马蹄下，翅膀伸展；底部 exergue 内镌 1887；Pistrucci 经典马剑图</t>
+          <t>背面: 圣乔治策马刺剑,斗篷飞扬,长矛刺杀毒龙,骏马前蹄腾空;龙蜷于马蹄下,翅膀伸展;底部 exergue 内镌 1887;Pistrucci 经典马剑图</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1898,12 +1898,12 @@
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>维多利亚女王禧年（Jubilee Head）是1887年为纪念女王登基50周年而发行的纪念性头像。5克劳恩（5 shillings = 1 Crown）是英国高价值银币，由皇家造币厂铸造。禧年头像由雕塑家约瑟夫·爱德华·伯姆（Joseph Edgar Boehm）设计，是维多利亚时代最具辨识度的钱币肖像之一。</t>
+          <t>维多利亚女王禧年(Jubilee Head)是1887年为纪念女王登基50周年而发行的纪念性头像。5克劳恩(5 shillings = 1 Crown)是英国高价值银币,由皇家造币厂铸造。禧年头像由雕塑家约瑟夫·爱德华·伯姆(Joseph Edgar Boehm)设计,是维多利亚时代最具辨识度的钱币肖像之一。</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -2001,12 +2001,12 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>保罗·冯·兴登堡（Paul von Hindenburg，1847-1934）是德国著名军事将领和政治家，于1925年至1934年担任魏玛共和国总统。1933年他任命阿道夫·希特勒为总理，最终导致纳粹党掌权。&lt;br&gt;&lt;br&gt;"Reichsadler"（帝国之鹰）版5马克银币正面为兴登堡戎装胸像，背面为德意志帝国之鹰纹章。这类银币是魏玛共和国末期的重要流通货币，1938年铸造版见证了第三帝国早期的经济与货币体系。A标表示由柏林造币厂（Berlin）铸造。</t>
+          <t>保罗·冯·兴登堡(Paul von Hindenburg,1847-1934)是德国著名军事将领和政治家,于1925年至1934年担任魏玛共和国总统。1933年他任命阿道夫·希特勒为总理,最终导致纳粹党掌权。&lt;br&gt;&lt;br&gt;"Reichsadler"(帝国之鹰)版5马克银币正面为兴登堡戎装胸像,背面为德意志帝国之鹰纹章。这类银币是魏玛共和国末期的重要流通货币,1938年铸造版见证了第三帝国早期的经济与货币体系。A标表示由柏林造币厂(Berlin)铸造。</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -2048,7 +2048,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2104,12 +2104,12 @@
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>保罗·冯·兴登堡（Paul von Hindenburg，1847-1934）是德国著名军事将领和政治家，于1925年至1934年担任魏玛共和国总统。1933年他任命阿道夫·希特勒为总理，最终导致纳粹党掌权。&lt;br&gt;&lt;br&gt;"Reichsadler"（帝国之鹰）版5马克银币正面为兴登堡戎装胸像，背面为德意志帝国之鹰纹章。这类银币是魏玛共和国末期至第三帝国早期的重要流通货币，1938年铸造版见证了战前德国的货币体系。A标表示由柏林造币厂（Berlin）铸造。</t>
+          <t>保罗·冯·兴登堡(Paul von Hindenburg,1847-1934)是德国著名军事将领和政治家,于1925年至1934年担任魏玛共和国总统。1933年他任命阿道夫·希特勒为总理,最终导致纳粹党掌权。&lt;br&gt;&lt;br&gt;"Reichsadler"(帝国之鹰)版5马克银币正面为兴登堡戎装胸像,背面为德意志帝国之鹰纹章。这类银币是魏玛共和国末期至第三帝国早期的重要流通货币,1938年铸造版见证了战前德国的货币体系。A标表示由柏林造币厂(Berlin)铸造。</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>正面: 蛇正从篮中爬出，周围常春藤花环环绕，花叶饱满</t>
+          <t>正面: 蛇正从篮中爬出,周围常春藤花环环绕,花叶饱满</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2217,12 +2217,12 @@
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>蛇篮（Cista Mystica）是古希腊祭祀酒神狄奥尼索斯仪式中的神圣器物——一个装有幼蛇的柳编篮子，祭司将其取出让蛇爬出，以此象征神迹与重生。这一意象被广泛铸造在银币背面，成为古希腊钱币中最具神秘感的经典图式。此币正面蛇从篮中爬出，周围常春藤花环环绕；背面双蛇缠绕弓箭袋，铭文「AΠOΛΛΩNIOΣ ΕΥΑΡΧΟΥ」清晰漂亮——地方行政官阿波罗尼奥斯，尤阿尔科斯之子。公元前133年帕加马王国灭亡，小亚细亚落入罗马人之手，此币恐由罗马总督发行，兑换比率为三枚狄纳里银币换一枚蛇篮四德拉克马。</t>
+          <t>蛇篮(Cista Mystica)是古希腊祭祀酒神狄奥尼索斯仪式中的神圣器物--一个装有幼蛇的柳编篮子,祭司将其取出让蛇爬出,以此象征神迹与重生。这一意象被广泛铸造在银币背面,成为古希腊钱币中最具神秘感的经典图式。此币正面蛇从篮中爬出,周围常春藤花环环绕;背面双蛇缠绕弓箭袋,铭文「AΠOΛΛΩNIOΣ ΕΥΑΡΧΟΥ」清晰漂亮--地方行政官阿波罗尼奥斯,尤阿尔科斯之子。公元前133年帕加马王国灭亡,小亚细亚落入罗马人之手,此币恐由罗马总督发行,兑换比率为三枚狄纳里银币换一枚蛇篮四德拉克马。</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>正面: 珀尔修斯右向头像，戴弗里吉亚帽（狮鹫装饰）；Aegis 护符</t>
+          <t>正面: 珀尔修斯右向头像,戴弗里吉亚帽(狮鹫装饰);Aegis 护符</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>背面: ΑΜΙΣΟΥ · 飞马 Pegasus 左向饮水；exergue 内徽记</t>
+          <t>背面: ΑΜΙΣΟΥ · 飞马 Pegasus 左向饮水;exergue 内徽记</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2330,12 +2330,12 @@
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>本都（Pontus）是黑海南岸的希腊化王国，以阿米索斯（Amisos，今土耳其Samsun）为重要造币与商业中心。米特拉达梯六世（&lt;b&gt;Mithradates VI Eupator&lt;/b&gt;，约 120-63 BC）是本都最伟大的国王，史称"米特拉达梯大帝"——先后三次发动对罗马的战争（前 88-前 63 年"米特拉达梯战争"），一度征服小亚细亚、希腊和爱琴海诸岛，几乎推翻罗马在东方的霸权。最终被庞培击败，逃往克里米亚后自杀。&lt;br&gt;&lt;br&gt;此币的&lt;b&gt;珀尔修斯戴弗里吉亚帽（Pileus / Phrygian cap）&lt;/b&gt;形象有强烈的政治神话含义：米特拉达梯王室自诩为希腊英雄珀尔修斯（斩杀美杜莎、救赎安德洛墨达）后裔——珀尔修斯之子&lt;b&gt;Perses&lt;/b&gt;被认为波斯与本都王族的始祖。弗里吉亚帽在希腊罗马语境中象征&lt;b&gt;自由&lt;/b&gt;，而帽上的&lt;b&gt;狮鹫装饰（griffin-crest）&lt;/b&gt;则呼应波斯/东方传统，体现米特拉达梯横跨东西方的统治合法性。&lt;br&gt;&lt;br&gt;背面的&lt;b&gt;飞马 Pegasus&lt;/b&gt;是阿米索斯建城神话的核心元素（飞马用蹄踢出 Hippene 泉），也是该城数百年来的固定币面主题。这枚铜币是希腊化王国政治宣传与地方传统结合的典型样本。</t>
+          <t>本都(Pontus)是黑海南岸的希腊化王国,以阿米索斯(Amisos,今土耳其Samsun)为重要造币与商业中心。米特拉达梯六世(&lt;b&gt;Mithradates VI Eupator&lt;/b&gt;,约 120-63 BC)是本都最伟大的国王,史称"米特拉达梯大帝"--先后三次发动对罗马的战争(前 88-前 63 年"米特拉达梯战争"),一度征服小亚细亚、希腊和爱琴海诸岛,几乎推翻罗马在东方的霸权。最终被庞培击败,逃往克里米亚后自杀。&lt;br&gt;&lt;br&gt;此币的&lt;b&gt;珀尔修斯戴弗里吉亚帽(Pileus / Phrygian cap)&lt;/b&gt;形象有强烈的政治神话含义:米特拉达梯王室自诩为希腊英雄珀尔修斯(斩杀美杜莎、救赎安德洛墨达)后裔--珀尔修斯之子&lt;b&gt;Perses&lt;/b&gt;被认为波斯与本都王族的始祖。弗里吉亚帽在希腊罗马语境中象征&lt;b&gt;自由&lt;/b&gt;,而帽上的&lt;b&gt;狮鹫装饰(griffin-crest)&lt;/b&gt;则呼应波斯/东方传统,体现米特拉达梯横跨东西方的统治合法性。&lt;br&gt;&lt;br&gt;背面的&lt;b&gt;飞马 Pegasus&lt;/b&gt;是阿米索斯建城神话的核心元素(飞马用蹄踢出 Hippene 泉),也是该城数百年来的固定币面主题。这枚铜币是希腊化王国政治宣传与地方传统结合的典型样本。</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>正面: 阿波罗·卡内奥斯（Apollo Carneius）侧面头像 · 年轻俊美 · 羊角与桂冠共存</t>
+          <t>正面: 阿波罗·卡内奥斯(Apollo Carneius)侧面头像 · 年轻俊美 · 羊角与桂冠共存</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2443,12 +2443,12 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>昔兰尼（Cyrenaica，今利比亚东部）于公元前631年建城，相传由一群来自帖飞的移民在阿波罗神谕指引下建立。此城迅速崛起为古代世界最富庶的城邦之一，全赖一种神奇植物——Silphium（又名忘忧草， Laserpitium silphium）。这种形似巨大茴香的伞形科植物，只生长在昔兰尼周边海岸，拥有令人惊叹的医疗功效，尤其以高效的避孕作用闻名——古代妇女将其汁液涂抹于子宫口，成功率接近百分之百。其贸易价值极高，一磅Silphium的价格相当于一个罗马士兵六年的薪俸，罗马元老院甚至在其铸造的银币上压制Silphium图案，作为帝国繁荣的象征。塞琉古帝国在公元前3世纪初攻占昔兰尼后废止本地铸币，此币发行于城市沦陷后的罗马统治早期，由当地官员以原塞琉古模具或本地模具发行，正面阿波罗·卡内奥斯（Apollo Carneius，羊角神）头像，羊角与桂冠共存，象征城邦保护神的神圣权威；背面Silphium枝叶繁茂，茎粗壮有力，果实心脏形，根系卷曲——这一经典图式在昔兰尼钱币上延续了两百余年。令人唏嘘的是，公元1世纪Silphium已彻底灭绝，原因可能是过度采集、地震破坏与土壤退化三重打击。</t>
+          <t>昔兰尼(Cyrenaica,今利比亚东部)于公元前631年建城,相传由一群来自帖飞的移民在阿波罗神谕指引下建立。此城迅速崛起为古代世界最富庶的城邦之一,全赖一种神奇植物--Silphium(又名忘忧草, Laserpitium silphium)。这种形似巨大茴香的伞形科植物,只生长在昔兰尼周边海岸,拥有令人惊叹的医疗功效,尤其以高效的避孕作用闻名--古代妇女将其汁液涂抹于子宫口,成功率接近百分之百。其贸易价值极高,一磅Silphium的价格相当于一个罗马士兵六年的薪俸,罗马元老院甚至在其铸造的银币上压制Silphium图案,作为帝国繁荣的象征。塞琉古帝国在公元前3世纪初攻占昔兰尼后废止本地铸币,此币发行于城市沦陷后的罗马统治早期,由当地官员以原塞琉古模具或本地模具发行,正面阿波罗·卡内奥斯(Apollo Carneius,羊角神)头像,羊角与桂冠共存,象征城邦保护神的神圣权威;背面Silphium枝叶繁茂,茎粗壮有力,果实心脏形,根系卷曲--这一经典图式在昔兰尼钱币上延续了两百余年。令人唏嘘的是,公元1世纪Silphium已彻底灭绝,原因可能是过度采集、地震破坏与土壤退化三重打击。</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>背面: 丰饶角两侧为狄俄斯库里兄弟皮里帽，ΑΜΙ-ΣΟΥ横列下方</t>
+          <t>背面: 丰饶角两侧为狄俄斯库里兄弟皮里帽,ΑΜΙ-ΣΟΥ横列下方</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2556,12 +2556,12 @@
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>本都王国（Pontos）位于安纳托利亚北部黑海沿岸，阿米索斯（Amisos，今土耳其萨姆松）是其最重要的港口城市之一。本都王国自米特里达梯一世建立，经历了数代君主的统治。约BC 120年，米特里达梯六世（Mithradates VI Eupator）继位，由于年幼由母亲摄政，此枚铜币即发行于这一时期。丰饶角象征富饶，狄俄斯库里兄弟的双帽子则暗示港口的航海保护，八芒星则代表这对孪生神兄弟。铭文ΑΜΙΣΟΥ即阿米索斯的希腊文拼写。</t>
+          <t>本都王国(Pontos)位于安纳托利亚北部黑海沿岸,阿米索斯(Amisos,今土耳其萨姆松)是其最重要的港口城市之一。本都王国自米特里达梯一世建立,经历了数代君主的统治。约BC 120年,米特里达梯六世(Mithradates VI Eupator)继位,由于年幼由母亲摄政,此枚铜币即发行于这一时期。丰饶角象征富饶,狄俄斯库里兄弟的双帽子则暗示港口的航海保护,八芒星则代表这对孪生神兄弟。铭文ΑΜΙΣΟΥ即阿米索斯的希腊文拼写。</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:18</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -2674,12 +2674,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-07T17:45:09</t>
-        </is>
-      </c>
-      <c r="Z20" t="inlineStr">
-        <is>
-          <t>b3a8a12</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -2726,7 +2721,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2736,12 +2731,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>正面: 戴维露姆面纱的君士坦丁一世半身像向右 · 铭文 DV CONSTANTINVS PT AVGG（神化君主君士坦丁，诸帝之父）</t>
+          <t>正面: 戴维露姆面纱的君士坦丁一世半身像向右 · 铭文 DV CONSTANTINVS PT AVGG(神化君主君士坦丁,诸帝之父)</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>背面: 君士坦丁穿托加盖头之站姿全身像 · 铭文 VN - MR（Veneranda Memoria 应受崇敬之记忆）· 底注 CONST（君士坦丁堡造币厂）</t>
+          <t>背面: 君士坦丁穿托加盖头之站姿全身像 · 铭文 VN - MR(Veneranda Memoria 应受崇敬之记忆)· 底注 CONST(君士坦丁堡造币厂)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2787,12 +2782,12 @@
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>公元337年5月22日，君士坦丁大帝（Constantinus I，公元306-337年在位）在尼科米底亚驾崩，结束了对罗马帝国近三十年的统治。这位在位期间颁布《米兰敕令》（313年）、召开尼西亚公会议（325年）、迁都博斯普鲁斯海峡并以「新罗马」命名新都的皇帝，是罗马世界最具变革意义的统治者之一。 君士坦丁驾崩后，其三位子嗣——君士坦丁二世、君士坦提乌斯二世、君士坦斯——共同继承帝位，史称「三兄共治」（337-340年）。按照罗马传统，前任皇帝在驾崩后即被元老院封神（Consecratio），纳入罗马神祇之列并享有祭祀。新任诸帝随即在各大造币厂发行追思币（Memorial Issue / Divus Issue），纪念亡父之「成神」，并以铭文宣告其「诸帝之父」（Pater Augustorum）的崇高地位。 此枚追思币为君士坦提乌斯二世（Constantius II，公元337-361年在位）在位初期所发行。正面铭文「DV CONSTANTINVS PT AVGG」——意即「神化君主君士坦丁，诸帝之父」——其中「PT」（Pater，之父）是追思币特有的称号，标明逝者为在位诸帝之父。戴维露姆面纱（velum）的半身像表明君士坦丁已被纳入神之行列。**特别值得关注的是正面铭文采用「DV」而非常见的「DN」（Dominus Noster，吾主）**——此或为特定造币厂之变体写法，亦可能因实物磨损导致字母辨识存疑，故仍以实物记录为准。 背面的「VN-MR」铭文实为「Veneranda Memoria」（应受崇敬之记忆）之缩写，是君士坦丁追思币中**特殊变体类型**之一。相较于更为常见的「CONS（Consecratio）」型封神图案（祭坛配阶梯），VN-MR型以**戴面纱穿托加的君士坦丁站姿全身像**为核心，配合「应受崇敬之记忆」的铭文，传达对已故君主的永恒怀念。底注「CONST」指示该币铸造于**君士坦丁堡造币厂**（Constantinople Mint），即君士坦丁大帝亲手建立的新都城。</t>
+          <t>公元337年5月22日,君士坦丁大帝(Constantinus I,公元306-337年在位)在尼科米底亚驾崩,结束了对罗马帝国近三十年的统治。这位在位期间颁布《米兰敕令》(313年)、召开尼西亚公会议(325年)、迁都博斯普鲁斯海峡并以「新罗马」命名新都的皇帝,是罗马世界最具变革意义的统治者之一。 君士坦丁驾崩后,其三位子嗣--君士坦丁二世、君士坦提乌斯二世、君士坦斯--共同继承帝位,史称「三兄共治」(337-340年)。按照罗马传统,前任皇帝在驾崩后即被元老院封神(Consecratio),纳入罗马神祇之列并享有祭祀。新任诸帝随即在各大造币厂发行追思币(Memorial Issue / Divus Issue),纪念亡父之「成神」,并以铭文宣告其「诸帝之父」(Pater Augustorum)的崇高地位。 此枚追思币为君士坦提乌斯二世(Constantius II,公元337-361年在位)在位初期所发行。正面铭文「DV CONSTANTINVS PT AVGG」--意即「神化君主君士坦丁,诸帝之父」--其中「PT」(Pater,之父)是追思币特有的称号,标明逝者为在位诸帝之父。戴维露姆面纱(velum)的半身像表明君士坦丁已被纳入神之行列。**特别值得关注的是正面铭文采用「DV」而非常见的「DN」(Dominus Noster,吾主)**--此或为特定造币厂之变体写法,亦可能因实物磨损导致字母辨识存疑,故仍以实物记录为准。 背面的「VN-MR」铭文实为「Veneranda Memoria」(应受崇敬之记忆)之缩写,是君士坦丁追思币中**特殊变体类型**之一。相较于更为常见的「CONS(Consecratio)」型封神图案(祭坛配阶梯),VN-MR型以**戴面纱穿托加的君士坦丁站姿全身像**为核心,配合「应受崇敬之记忆」的铭文,传达对已故君主的永恒怀念。底注「CONST」指示该币铸造于**君士坦丁堡造币厂**(Constantinople Mint),即君士坦丁大帝亲手建立的新都城。</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:18</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2834,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2849,12 +2844,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>正面: 哈德良面向右之桂冠胸像 · 赤膊上身，左肩披托加 · 铭文 IMP CAESAR TRAIANVS HADRIANVS AVG</t>
+          <t>正面: 哈德良面向右之桂冠胸像 · 赤膊上身,左肩披托加 · 铭文 IMP CAESAR TRAIANVS HADRIANVS AVG</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>背面: 赏赐场景（Congiarium）——皇帝坐高台折叠椅面左，右手前伸；助手向台下公民分发赏赐；Liberalitas女神站于背景持钱袋 · 铭文 PONT MAX TR POT COS II / LIBERALITAS AVG / SC</t>
+          <t>背面: 赏赐场景(Congiarium)--皇帝坐高台折叠椅面左,右手前伸;助手向台下公民分发赏赐;Liberalitas女神站于背景持钱袋 · 铭文 PONT MAX TR POT COS II / LIBERALITAS AVG / SC</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2900,12 +2895,12 @@
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>在古罗马，有一种特殊的活动叫congiarium，起初它是向罗马城市居民分发油或酒，到奥古斯都时期演变成了在特殊场合（如皇帝登基、庆祝凯旋等）分发钱财。从尼禄统治时期开始，钱币上就出现了congiarium的场景，画面中总有一个人高举着带长柄的矩形物体。而当「慷慨」（Liberalitas）这一拟人形象在哈德良统治时期首次出现在钱币上时，这个矩形物体成了她的标志性特征。 这个神秘的矩形物体到底是什么呢？此前有多种解读。有人认为它是「tessera」（一种代币或凭证），也有人觉得是「abacus」（算盘），但观察不同皇帝时期钱币上对congiarium仪式图案的演变，尼禄时期的钱币上有两种图案形式，一种成了后续皇帝钱币的标准样式；图拉真时期的图案似乎印证congiarium有两个阶段；哈德良时期，「慷慨」拟人形象出现，逐渐取代了原本拿着矩形物体的男性形象。 结合历史记载中 congiarium 发放的货币面额信息（大多为第纳里乌斯银币，有时也会使用奥里斯金币），这个矩形物体极有可能是用于分发钱币的计数板。其表面的圆形凹陷，可辅助工作人员迅速数出待分发的钱币数量。在君士坦丁凯旋门的浮雕上，我们能够清晰看到皇帝使用类似物体向接受者分发钱币的场景。此外，画面中拿着它的人将其举到与头平齐或更高的位置展示给接受者和在场众人，保证分发过程的公平和诚实，避免出现盗窃和欺诈行为。 总的来说，这个成为「慷慨」拟人形象标志性特征的矩形物体，是congiarium仪式中不可或缺的计数、展示和分发工具，它在加快分发速度的同时，保障了分发的公正性。对于古罗马钱币收藏者而言，了解这些知识，能让我们手中的钱币「开口说话」，也是探索古罗马社会经济、政治和文化的重要线索。</t>
+          <t>在古罗马,有一种特殊的活动叫congiarium,起初它是向罗马城市居民分发油或酒,到奥古斯都时期演变成了在特殊场合(如皇帝登基、庆祝凯旋等)分发钱财。从尼禄统治时期开始,钱币上就出现了congiarium的场景,画面中总有一个人高举着带长柄的矩形物体。而当「慷慨」(Liberalitas)这一拟人形象在哈德良统治时期首次出现在钱币上时,这个矩形物体成了她的标志性特征。 这个神秘的矩形物体到底是什么呢?此前有多种解读。有人认为它是「tessera」(一种代币或凭证),也有人觉得是「abacus」(算盘),但观察不同皇帝时期钱币上对congiarium仪式图案的演变,尼禄时期的钱币上有两种图案形式,一种成了后续皇帝钱币的标准样式;图拉真时期的图案似乎印证congiarium有两个阶段;哈德良时期,「慷慨」拟人形象出现,逐渐取代了原本拿着矩形物体的男性形象。 结合历史记载中 congiarium 发放的货币面额信息(大多为第纳里乌斯银币,有时也会使用奥里斯金币),这个矩形物体极有可能是用于分发钱币的计数板。其表面的圆形凹陷,可辅助工作人员迅速数出待分发的钱币数量。在君士坦丁凯旋门的浮雕上,我们能够清晰看到皇帝使用类似物体向接受者分发钱币的场景。此外,画面中拿着它的人将其举到与头平齐或更高的位置展示给接受者和在场众人,保证分发过程的公平和诚实,避免出现盗窃和欺诈行为。 总的来说,这个成为「慷慨」拟人形象标志性特征的矩形物体,是congiarium仪式中不可或缺的计数、展示和分发工具,它在加快分发速度的同时,保障了分发的公正性。对于古罗马钱币收藏者而言,了解这些知识,能让我们手中的钱币「开口说话」,也是探索古罗马社会经济、政治和文化的重要线索。</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:18</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -2962,12 +2957,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>正面: 戴头盔的罗马女神（Roma）左侧胸像，手持盾牌，长矛扛于肩后。</t>
+          <t>正面: 戴头盔的罗马女神(Roma)左侧胸像,手持盾牌,长矛扛于肩后。</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>背面: X / P·NERVA，两名公民在公民大会广场（comitium）投票，左侧公民手持选票板（tabella），右侧公民将选票投入开启的投票箱（cista）。底部横线装饰（a line of dots）。</t>
+          <t>背面: X / P·NERVA,两名公民在公民大会广场(comitium)投票,左侧公民手持选票板(tabella),右侧公民将选票投入开启的投票箱(cista)。底部横线装饰(a line of dots)。</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3018,12 +3013,12 @@
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>这是罗马共和国晚期最著名的投票场景德纳里乌斯之一，由造币三巨头（tresvir monetalis）P. Licinius Nerva 于公元前113-112年铸造。 背面所描叙的公民投票场景是罗马共和政治史中极其罕见的图像记录：一名选民从下方助手手中接过选票（tabella），另一名选民将选票投入票箱（cista），右上方有一张标有字母P的选票。 这一图景与罗马秘密投票制（tabella）的历史性改革密切相关。公元前139年的 Lex Gabinia 引入了立法大会中的无记名投票，公元前137年的 Lex Cassia 将其扩展至司法审判，公元前131年的 Lex Papiria 进一步强化其适用。这一系列改革标志着罗马民主程序的重要进化——公民不再需要公开自己的投票立场。 选票上的P字学界通常解释为某位候选人姓名的首字母缩写，具体指代仍有争议。 P. Licinius Nerva 出身李锡尼亚氏族（gens Licinia），其本身日后也成为罗马政坛重要人物。</t>
+          <t>这是罗马共和国晚期最著名的投票场景德纳里乌斯之一,由造币三巨头(tresvir monetalis)P. Licinius Nerva 于公元前113-112年铸造。 背面所描叙的公民投票场景是罗马共和政治史中极其罕见的图像记录:一名选民从下方助手手中接过选票(tabella),另一名选民将选票投入票箱(cista),右上方有一张标有字母P的选票。 这一图景与罗马秘密投票制(tabella)的历史性改革密切相关。公元前139年的 Lex Gabinia 引入了立法大会中的无记名投票,公元前137年的 Lex Cassia 将其扩展至司法审判,公元前131年的 Lex Papiria 进一步强化其适用。这一系列改革标志着罗马民主程序的重要进化--公民不再需要公开自己的投票立场。 选票上的P字学界通常解释为某位候选人姓名的首字母缩写,具体指代仍有争议。 P. Licinius Nerva 出身李锡尼亚氏族(gens Licinia),其本身日后也成为罗马政坛重要人物。</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:18</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3065,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -3080,12 +3075,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>正面: 拿破仑面向左之桂冠头像 · 铭文 NAPOLEONE IMPERATORE E RE（拿破仑皇帝兼国王）· 底部署名 1811 · 造币厂标记 M（Milano，米兰）</t>
+          <t>正面: 拿破仑面向左之桂冠头像 · 铭文 NAPOLEONE IMPERATORE E RE(拿破仑皇帝兼国王)· 底部署名 1811 · 造币厂标记 M(Milano,米兰)</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>背面: 伦巴第铁王冠（Lombardy Iron Crown）· 顶部铭文 REGNO D'ITALIA（意大利王国）· 底部面值 1 SOLDO</t>
+          <t>背面: 伦巴第铁王冠(Lombardy Iron Crown)· 顶部铭文 REGNO D'ITALIA(意大利王国)· 底部面值 1 SOLDO</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3131,12 +3126,12 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>1811年拿破仑帝国鼎盛时期，意大利王国（Regno d'Italia）铸造的1索尔迪铜币。米兰造币厂（Mint Mark M）出品，编号NGC-AU50，成交价992元，来源云台主人2025年10月。 拿破仑于1805年在米兰加冕为意大利国王，随后在意大利领土上推行与法兰西帝国一致的行政、金融与货币体系。意大利王国使用法国货币标准：里拉（Lira）为记账单位，辅币包括索尔迪（Soldo，1里拉=20索尔迪）和分（Centesimo，1索尔迪=5分）。此枚1索尔迪铜币正面为拿破仑桂冠头像，铭文NAPOLEONE IMPERATORE E RE（拿破仑皇帝兼国王），底部署名1811与造币厂标记M（Milano）。背面为伦巴第铁王冠（Lombardy Iron Crown）——意大利统一运动的核心象征，王冠中心铭刻REGNO D'ITALIA（意大利王国），底部面值1 SOLDO。 伦巴第铁王冠（Lombardy Iron Crown）相传以钉死耶稣的圣钉铸造，直径4.5厘米，重约250克，外包金箔，内环为铁质。它是中世纪伦巴第王国及意大利独立运动的重要象征，拿破仑在取得马伦戈战役（1800年）后于伦巴第加冕时使用过此王冠。将铁王冠图案铸于钱币，既是拿破仑宣示其意大利王权的政治行为，也暗示他继承了意大利乃至神圣罗马帝国的历史正统性。此币NGC AU50品相，币面光亮，边齿锐利，是意大利王国拿破仑时期铜币的典型收藏品。</t>
+          <t>1811年拿破仑帝国鼎盛时期,意大利王国(Regno d'Italia)铸造的1索尔迪铜币。米兰造币厂(Mint Mark M)出品,编号NGC-AU50,成交价992元,来源云台主人2025年10月。 拿破仑于1805年在米兰加冕为意大利国王,随后在意大利领土上推行与法兰西帝国一致的行政、金融与货币体系。意大利王国使用法国货币标准:里拉(Lira)为记账单位,辅币包括索尔迪(Soldo,1里拉=20索尔迪)和分(Centesimo,1索尔迪=5分)。此枚1索尔迪铜币正面为拿破仑桂冠头像,铭文NAPOLEONE IMPERATORE E RE(拿破仑皇帝兼国王),底部署名1811与造币厂标记M(Milano)。背面为伦巴第铁王冠(Lombardy Iron Crown)--意大利统一运动的核心象征,王冠中心铭刻REGNO D'ITALIA(意大利王国),底部面值1 SOLDO。 伦巴第铁王冠(Lombardy Iron Crown)相传以钉死耶稣的圣钉铸造,直径4.5厘米,重约250克,外包金箔,内环为铁质。它是中世纪伦巴第王国及意大利独立运动的重要象征,拿破仑在取得马伦戈战役(1800年)后于伦巴第加冕时使用过此王冠。将铁王冠图案铸于钱币,既是拿破仑宣示其意大利王权的政治行为,也暗示他继承了意大利乃至神圣罗马帝国的历史正统性。此币NGC AU50品相,币面光亮,边齿锐利,是意大利王国拿破仑时期铜币的典型收藏品。</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:18</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3193,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>背面: 海鹰展开双翅向左飞行抓握海豚 · 底部铭文 IΣTPIH（Istros，伊斯特罗斯）</t>
+          <t>背面: 海鹰展开双翅向左飞行抓握海豚 · 底部铭文 IΣTPIH(Istros,伊斯特罗斯)</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3244,12 +3239,12 @@
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>莫西亚（Moesia）伊斯特罗斯（Istros，黑海西岸重要城邦，约今罗马尼亚境内多瑙河三角洲）铸造的古典银币。 正面为双少年头像——一正一反、相互环绕。这种独特的双人头像图案是伊斯特罗斯城币的标志性设计，其象征意义学界尚有争议：一种观点认为代表Dioscuri（双子神卡斯托尔与波吕克斯），另一观点认为表现城邦的两位创建英雄或神灵（Heroes）。 背面为海鹰（鸥鹭）展开双翅抓握海豚，向左飞行。底部署名IΣTPIH（伊斯特罗斯城的希腊文名称）。这一图案反映了伊斯特罗斯作为黑海贸易港口的海洋经济特征——海鹰象征天空与神意，海豚象征海洋与商业繁荣，两者结合宣示城市对黑海贸易通道的掌控。 伊斯特罗斯城约公元前656年由米勒图斯（Miletus）移民建立，是黑海地区最早的希腊殖民城邦之一。其钱币铸造传统延续数百年，银币体系与雅典、爱奥尼亚等地有密切往来。</t>
+          <t>莫西亚(Moesia)伊斯特罗斯(Istros,黑海西岸重要城邦,约今罗马尼亚境内多瑙河三角洲)铸造的古典银币。 正面为双少年头像--一正一反、相互环绕。这种独特的双人头像图案是伊斯特罗斯城币的标志性设计,其象征意义学界尚有争议:一种观点认为代表Dioscuri(双子神卡斯托尔与波吕克斯),另一观点认为表现城邦的两位创建英雄或神灵(Heroes)。 背面为海鹰(鸥鹭)展开双翅抓握海豚,向左飞行。底部署名IΣTPIH(伊斯特罗斯城的希腊文名称)。这一图案反映了伊斯特罗斯作为黑海贸易港口的海洋经济特征--海鹰象征天空与神意,海豚象征海洋与商业繁荣,两者结合宣示城市对黑海贸易通道的掌控。 伊斯特罗斯城约公元前656年由米勒图斯(Miletus)移民建立,是黑海地区最早的希腊殖民城邦之一。其钱币铸造传统延续数百年,银币体系与雅典、爱奥尼亚等地有密切往来。</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:18</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -3291,7 +3286,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -3347,12 +3342,12 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>阿斯潘多斯（Aspendos）是潘菲利亚（Pamphylia）地区最重要的希腊殖民城市之一，位于欧里梅顿河（Eurymedon）入海口附近。该城在公元前 5 世纪波斯统治时期及随后的希腊化时期始终保持高度自治权，其独特的货币体系在整个安纳托利亚南部具有代表性。&lt;br&gt;&lt;br&gt;阿斯潘多斯银币正面描绘两名摔跤手（wrestlers）正在进行角力比赛——这是古希腊体育竞技（pankration 或 wrestling）的经典题材，可能与当地举办的运动赛事或狄奥斯库里（Dockeroi）的神话典故有关。两摔跤手之间的 "FK" 是造币厂缩写或工匠标记。&lt;br&gt;&lt;br&gt;背面描绘一名投石手（slinger）向右行走，正准备发射投石弹丸（bullet）。投石兵是安纳托利亚南部轻装步兵的典型代表，该形象可能与当地军事传统或赫拉克勒斯使用投石带的神话主题有关。三曲腿图（triskeles）是阿斯潘多斯币的典型辅助符号。铭文 "EΣTFEΔΙΙΥΣ" 是阿斯潘多斯（Aspendos）的希腊语城市名，置于颗粒方框（pellet square）内是潘菲利亚地区造币的典型边框设计。SNG France 103 将该版式归为阿斯潘多斯古典晚期（约 BC 380-325）标准银币。币面投石手下方有小凹痕（small ding below slinger）。</t>
+          <t>阿斯潘多斯(Aspendos)是潘菲利亚(Pamphylia)地区最重要的希腊殖民城市之一,位于欧里梅顿河(Eurymedon)入海口附近。该城在公元前 5 世纪波斯统治时期及随后的希腊化时期始终保持高度自治权,其独特的货币体系在整个安纳托利亚南部具有代表性。&lt;br&gt;&lt;br&gt;阿斯潘多斯银币正面描绘两名摔跤手(wrestlers)正在进行角力比赛--这是古希腊体育竞技(pankration 或 wrestling)的经典题材,可能与当地举办的运动赛事或狄奥斯库里(Dockeroi)的神话典故有关。两摔跤手之间的 "FK" 是造币厂缩写或工匠标记。&lt;br&gt;&lt;br&gt;背面描绘一名投石手(slinger)向右行走,正准备发射投石弹丸(bullet)。投石兵是安纳托利亚南部轻装步兵的典型代表,该形象可能与当地军事传统或赫拉克勒斯使用投石带的神话主题有关。三曲腿图(triskeles)是阿斯潘多斯币的典型辅助符号。铭文 "EΣTFEΔΙΙΥΣ" 是阿斯潘多斯(Aspendos)的希腊语城市名,置于颗粒方框(pellet square)内是潘菲利亚地区造币的典型边框设计。SNG France 103 将该版式归为阿斯潘多斯古典晚期(约 BC 380-325)标准银币。币面投石手下方有小凹痕(small ding below slinger)。</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -3394,12 +3389,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -3414,7 +3409,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>背面: 宙斯持鹰坐像 · ΑΛΕΞΑΝΔΡΟΥ（亚历山大的）</t>
+          <t>背面: 宙斯持鹰坐像 · ΑΛΕΞΑΝΔΡΟΥ(亚历山大的)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3460,12 +3455,12 @@
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>亚历山大三世（大帝，356-323 BC）统一希腊、征服波斯，建立了人类历史上第一个横跨欧亚非的超级帝国。他对货币体系的改革影响深远：四德拉克马银币以赫拉克勒斯头像为正面，宙斯持鹰坐像为背面，成为帝国扩张的战略工具与文化符号。随着亚历山大的征服，这套币制被推广至从埃及到印度河的广大地区，继业者纷纷仿铸。利西普斯（ Lysippos ）风格的赫拉克勒斯肖像极具古典理想美，而宙斯坐像手持雄鹰的形象则强化了王权的神圣性。此枚米勒都斯（Miletus）铸币约 BC 325-320 年所见宙斯底座无碑铭，为亚历山大在世时期的早期铸型。</t>
+          <t>亚历山大三世(大帝,356-323 BC)统一希腊、征服波斯,建立了人类历史上第一个横跨欧亚非的超级帝国。他对货币体系的改革影响深远:四德拉克马银币以赫拉克勒斯头像为正面,宙斯持鹰坐像为背面,成为帝国扩张的战略工具与文化符号。随着亚历山大的征服,这套币制被推广至从埃及到印度河的广大地区,继业者纷纷仿铸。利西普斯( Lysippos )风格的赫拉克勒斯肖像极具古典理想美,而宙斯坐像手持雄鹰的形象则强化了王权的神圣性。此枚米勒都斯(Miletus)铸币约 BC 325-320 年所见宙斯底座无碑铭,为亚历山大在世时期的早期铸型。</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:17</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -3568,12 +3563,12 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>此币正面图案献给 L. Cassius Longinus Ravilla——这位 L. Cassius Longinus（造币官）的祖父，他是一位备受尊敬的裁判官和法学家。公元前 113 年，Ravilla 主持了对三名维斯塔处女（Vestal Virgin）的审判，指控她们破坏贞操，最终判定其中两人有罪并处以死刑——这一事件在罗马历史上极为罕见，体现了罗马司法的严厉一面。他的银币背面所描绘的，正是他担任保民官期间（公元前 137 年）引入的罗马秘密投票制度的运作场景。这一制度革新标志着罗马公民无需在公开场合表明投票立场——投票权的引入深刻影响了罗马的民主进程。</t>
+          <t>此币正面图案献给 L. Cassius Longinus Ravilla--这位 L. Cassius Longinus(造币官)的祖父,他是一位备受尊敬的裁判官和法学家。公元前 113 年,Ravilla 主持了对三名维斯塔处女(Vestal Virgin)的审判,指控她们破坏贞操,最终判定其中两人有罪并处以死刑--这一事件在罗马历史上极为罕见,体现了罗马司法的严厉一面。他的银币背面所描绘的,正是他担任保民官期间(公元前 137 年)引入的罗马秘密投票制度的运作场景。这一制度革新标志着罗马公民无需在公开场合表明投票立场--投票权的引入深刻影响了罗马的民主进程。</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-07-07T17:23:18</t>
+          <t>2026-07-12T13:55:56</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3661,6 @@
           <t>2024-03</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr">
         <is>
           <t>2024</t>
@@ -3687,15 +3681,464 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-07-07T17:52:10</t>
-        </is>
-      </c>
-      <c r="Y29" t="inlineStr"/>
-      <c r="Z29" t="inlineStr">
-        <is>
-          <t>0555589</t>
-        </is>
-      </c>
+          <t>2026-07-12T13:55:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>GR-005</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CILICIA</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>塔苏斯 波斯总督银币</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>CILICIA · Tarsus · Mazaios (Satrap, BC 361-334)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>BC 361-334</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>1 Siglos 西格罗斯</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Silver 银 · 23.5mm · 10.8g</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>greek</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>正面: 巴力神坐像 (Baaltarses) · 右手托鹰 · 左手持莲花头权杖 · 阿拉米文 BLTRZ</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>背面: 狮子攻击公牛 · 阿拉米文 MZDI (马扎亚斯) · 下方 M · K 控制标记</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>西里西亚, 塔苏斯, 波斯总督, 西格罗斯</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>¥1,162</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>1162</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>良泉藏泉</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>images/GR-005.jpg</t>
+        </is>
+      </c>
+      <c r="V30" t="n">
+        <v>1868377</v>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>马扎亚斯（?-前328年），为波斯阿契美尼德帝国的贵族，也是大流士三世时的巴比伦尼亚总督。前331年，当亚历山大大帝东征时，马扎亚斯参与高加米拉战役，并且统帅波斯军队右翼，下辖叙利亚、米底、美索不达米亚、帕提亚、塔巴里斯坦、塞克(Saka)、赫卡尼亚、卡帕多细亚、阿尔巴尼亚等部队以及亚美尼亚骑兵。在战役中马扎亚斯借着人数优势，向马其顿左翼进行迂回，使马其顿左翼指挥官帕曼纽陷入困境，马扎亚斯几乎获得对马其顿左翼的胜利。但因亚历山大大帝率骑兵直接进入波斯军左翼的缺口，大流士三世落荒而逃，因发全军败退。马扎亚斯无法重整军队，才撤离战场。战后马扎亚斯向亚历山大献出巴比伦，亚历山大仍令他为巴比伦尼亚总督。马扎亚斯的未婚妻是大流士三世的女儿斯妲特拉二世，但斯妲特拉二世等大流士家眷在伊苏斯战役后沦为马其顿军的俘虏，加上马扎亚斯很早就去世，斯妲特拉二世便在苏萨集体婚礼中嫁给亚历山大大帝。&lt;br&gt;&lt;br&gt;巴力从叙利亚到波斯都有人崇拜，甚至在迦南文化中也有他的存在，希腊神话中，巴力转化为巴勒斯(Belos)，代表的即主神宙斯。其全称「巴力西卜」(Baal-zebul)本义为「天上的主人」，常简称为巴力(ba'al)，在旧约圣经中被多次提及，用「事奉巴力」一词描述离弃耶和华。以色列王亚哈的妻子耶洗别曾下令所有国民只能事奉巴力，并屠杀了耶和华的先知，新约中巴力已被丑化为鬼王别名。到了中世纪，巴力在所罗门的小钥匙中，成为七十二柱排第1位的魔王。巴耶力(Bael)以鬼王的名义指挥魔界66个军团守护四方。</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>2026-07-12T13:55:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>GK-013</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Indo-Greek Kingdom</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>希腊-巴克特里亚 · 阿波罗多托斯一世 Hemiobol 铜币</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Indo-Greek Kingdom · Apollodotus I (Σωτήρ)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>BC 174-165</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Hemiobol (1⁄12)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Copper · 25mm · 10.28g</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>SNG Copenhagen# 359</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>GK</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>正面: Apollo standing facing, holding arrow in right hand and bow in left; Greek legend on three sides</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>反面: Tripod within dotted border; monogram at right</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>GK, 阿波罗多托斯, 印度-希腊, 阿波罗, 三足祭坛</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>¥56</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>56</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>良泉藏泉</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>images/GK-013.jpg</t>
+        </is>
+      </c>
+      <c r="V31" t="n">
+        <v>2135645</v>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>阿波罗多托斯一世（'Aπολλόδοτος Α΄ ò Σωτήρ · 救主阿波罗多托斯，BC 186-160）是印度-希腊王国的开创君主之一，继承希腊-巴克特里亚王国南部领土后南下印度河流域创立王国。他发行的德拉克马银币和铜币以阿波罗形象为核心，正面为阿波罗立像手持弓箭，背面为德尔斐三足祭坛（τρίπους），象征阿波罗神职与希腊文化传统。希腊铭文使用「ΣΩΤΗΡ」（救主）称号，与塞琉古国王常用称号一致，旨在彰显其正统王权。佉卢文铭文则面向印度本地民众，体现希腊君主对当地文化习俗的包容与整合。此币面值 Hemiobol（1/12德拉克马），为日常小额交易所用铜币。</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>2026-07-12T13:55:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>NI-002</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Napoleone Imperatore e Re</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>意大利王国 · 拿破仑一世 5索尔迪 银币 1809 米兰</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Napoleone Imperatore e Re · Regno d'Italia · Milano</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>AD 1809</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>5 Soldi</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Silver · 15mm · 1.27g · 6h</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Mont. 279; KM 19/5.1; R1 (发行量602,134)</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>NI</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>正面: Tête nue de Napoléon Ier à droite / NAPOLEONE IMPERATORE E RE · 1809</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>反面: La Couronne de Fer / REGNO D'ITALIA · 5. SOLDI · M</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>NI, 拿破仑一世, 意大利王国, 5 Soldi, 铁王冠</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>€127</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>991</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>CGB</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>images/NI-002.jpg</t>
+        </is>
+      </c>
+      <c r="V32" t="n">
+        <v>190805</v>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>意大利王国（1805-1814）为拿破仑一世治下北意大利的附庸王国，由米兰总督区演化而来。1805年3月17日，拿破仑接受意大利王冠；5月26日，约瑟芬与他在米兰大教堂加冕，与巴黎加冕一样，他亲手将王冠戴上，宣告"上帝赐予我，触者当心"。后任命其女婿欧仁·德·博阿尔内为意大利总督。9年间，米兰造币厂以拿破仑名义发行全套意大利王国银铜币，5索尔迪为小额流通币，铁王冠（Corona di Ferro）作为王国主权标志，源自中世纪伦巴第王国。1814年1月缪拉背叛与奥地利结盟，意大利王国王朝崩溃。</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>2026-07-12T13:55:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>NI-003</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Napoleone Imperatore e Re</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>意大利王国 · 拿破仑一世 3 Centesimi 铜币 1813 米兰</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Napoleone Imperatore e Re · Regno d'Italia · Milano</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>AD 1813</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>3 Centesimi</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Copper · M</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Mont. 312</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>NI</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>正面: NAPOLEONE IMPERATORE E RE · Tête nue de Napoléon Ier à gauche · 1813 · M</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>反面: REGNO D'ITALIA · La Couronne de Fer · 3 CENTESIMI · M</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>NI, 拿破仑一世, 意大利王国, 3 Centesimi, 铁王冠</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>€96</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>749</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>CGB</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>images/NI-003.jpg</t>
+        </is>
+      </c>
+      <c r="V33" t="n">
+        <v>176279</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>意大利王国（1805-1814）为拿破仑一世治下北意大利的附庸王国。1813年铸造的3 Centesimi为该系列最后年份之一，1814年随着拿破仑第一次退位，意大利王国随之覆灭。铁王冠（Corona Ferrea）为伦巴第王国的古老加冕标志，也是拿破仑作为意大利国王的象征。</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>2026-07-12T13:55:56</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
新增 NI-004 意大利王国 1 Centesimo 1809 米兰 (CGB 2026-07)
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z33"/>
+  <dimension ref="A1:Z34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:55</t>
+          <t>2026-07-12T14:22:32</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:55</t>
+          <t>2026-07-12T14:22:32</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:32</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:32</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:32</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:32</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
+          <t>2026-07-12T14:22:33</t>
         </is>
       </c>
     </row>
@@ -4113,7 +4113,6 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr">
         <is>
           <t>2026</t>
@@ -4134,11 +4133,83 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-07-12T13:55:56</t>
-        </is>
-      </c>
-      <c r="Y33" t="inlineStr"/>
-      <c r="Z33" t="inlineStr"/>
+          <t>2026-07-12T14:22:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>NI-004</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Regno d'Italia</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Regno d'Italia · Napoléon I · 1 Centesimo · 1809 · Milano</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>AD 1809</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>拿破仑一世 Napoléon I Bonaparte</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>1 Centesimo 1 索尔多</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>铜 · Milano</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>NI</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>images/NI-004.jpg</t>
+        </is>
+      </c>
+      <c r="V34" t="n">
+        <v>144545</v>
+      </c>
+      <c r="W34" t="inlineStr"/>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>2026-07-12T14:22:33</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr"/>
+      <c r="Z34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add FM-002 法国古典式摔跤铜章 (R. Linzer)
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z37"/>
+  <dimension ref="A1:Z38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:25</t>
+          <t>2026-07-12T15:22:23</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:25</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:26</t>
+          <t>2026-07-12T15:22:24</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:27</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:27</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:27</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:27</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:27</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:27</t>
+          <t>2026-07-12T15:22:25</t>
         </is>
       </c>
     </row>
@@ -4565,7 +4565,6 @@
           <t>2024-07</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr">
         <is>
           <t>2024</t>
@@ -4586,11 +4585,125 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-07-12T15:17:27</t>
-        </is>
-      </c>
-      <c r="Y37" t="inlineStr"/>
-      <c r="Z37" t="inlineStr"/>
+          <t>2026-07-12T15:22:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>FM-002</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Lutte Gréco-Romaine</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>法国 · 古典式摔跤 铜质奖章</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Lutte Gréco-Romaine · Médaille de Bronze · R. Linzer</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>c. AD 1930–1950 (20 世纪上半叶)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>体育/摔跤奖章</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>铜 · 44.2mm · 42.8g · 红绿包浆</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>FM</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>正面: 两位裸体男子古典式摔跤(lutte gréco-romaine)扭打瞬间 · 高浮雕 · 底部双签名 E. KATZ (设计) / R. LINZER (雕刻)</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>反面: 月桂花环(couronne de laurier)围绕 · 中央空白留待后刻获奖者信息 · 底部丝带蝴蝶结收束</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>FM, 法国, 铜质奖章, 体育, 摔跤, 古典式, R. Linzer, 月桂花环</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>¥26</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>竞宝斋</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>images/FM-002.jpg</t>
+        </is>
+      </c>
+      <c r="V38" t="n">
+        <v>2938739</v>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>此为法国 20 世纪上半叶发行的体育奖章，正面表现古典式摔跤（lutte gréco-romaine）两位运动员的扭打瞬间。古典式摔跤是法国传统强项，19 世纪末在皮埃尔·德·顾拜旦（Pierre de Coubertin）推动现代奥运复兴后，该项目于 1896 年首届现代奥运会即被列入正式比赛。20 世纪上半叶法国各地摔跤俱乐部、博览会、工人体育联合会（Fédération Sportive du Travail）经常颁发此类奖章，以表彰比赛冠军与体育成就。&lt;br&gt;&lt;br&gt;本枚奖章由两位雕刻师合作完成：底部双签名 "E. KATZ"（设计师）与 "R. LINZER"（雕刻师）。R. LINZER 即 Robert Linzer（1901–1969），法国 20 世纪最重要的奖章雕刻师之一，曾长期任职于巴黎造币厂（Monnaie de Paris）的雕刻部门（Atelier de Gravure），为众多体育赛事、工业博览会、地方庆典雕刻奖章。其作品以高浮雕、动态人体刻画著称，古典美学与现代雕塑感并重。&lt;br&gt;&lt;br&gt;反面采用月桂花环（couronne de laurier）——这是源自古希腊罗马的胜利象征（corona triumphalis），是体育奖章与艺术奖章最常见的装饰母题。中央留白通常用于刻获奖者姓名、比赛名称、日期等铭文（此类后期铭刻因每枚奖章不同而通常未保留），底部以丝带蝴蝶结收束，是 20 世纪法国体育奖章的标准构图。&lt;br&gt;&lt;br&gt;章体红绿包浆（朱砂锈 + 绿锈）为铜质奖章历经数十年自然氧化的典型表现，虽有表面点状锈迹但整体浮雕完整，运动员肌肉、姿态、花环叶片均清晰可辨，是法国体育奖章艺术（Medallic Art）的实用物证。</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>2026-07-12T15:22:25</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr"/>
+      <c r="Z38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add FJ-005 Lyon Academie jeton 1749 D.V. (39 coins total)
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:17</t>
+          <t>2026-07-12T16:09:40</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:18</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:18</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:18</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:18</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:18</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:18</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:18</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:18</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:41</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:19</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:20</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:20</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr"/>
@@ -4814,7 +4814,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:20</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>FJ, 法国, 代用币, jeton, 银, 1750, 路易十五, 非凡战争, 闪电, 军事, R. Filius</t>
+          <t>FJ, 法国, 代用币, jeton, 银, 1750, 路易十五, 非凡战争, 闪电, 军事, R. Filius, 法国, 代用币, 里昂, 文学院, Jeton, FM, 法国, 银质奖章, 工业, 商会, 里尔, ROBERT, 950银</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4927,7 +4927,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:20</t>
+          <t>2026-07-12T16:09:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix FJ-005 card format: restore proper HTML comment structure (40 cards)
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z40"/>
+  <dimension ref="A1:Z41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:40</t>
+          <t>2026-07-12T16:22:08</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:41</t>
+          <t>2026-07-12T16:22:09</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4585,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-07-12T15:54:20</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr"/>
@@ -4814,7 +4814,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>FJ, 法国, 代用币, jeton, 银, 1750, 路易十五, 非凡战争, 闪电, 军事, R. Filius, 法国, 代用币, 里昂, 文学院, Jeton, FM, 法国, 银质奖章, 工业, 商会, 里尔, ROBERT, 950银</t>
+          <t>FJ, 法国, 代用币, jeton, 银, 1750, 路易十五, 非凡战争, 闪电, 军事, R. Filius</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -4927,7 +4927,75 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-07-12T16:09:42</t>
+          <t>2026-07-12T16:22:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>FJ-005</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>FJ</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>法国王室纹章（蓝底三朵百合花）置于纹章框内，两侧为里昂守护神——持桨的罗讷河神（DVX）与持立标的索恩河神（SAO）。</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>柱廊神庙，上方两位胜利女神持桂冠；铭文「ATHENAEUM LUGDUNENSE RESTITUTUM」（里昂文学院重建），年铭「ACADEM. LITTER. LUGDUN. MDCCXLIX」（MDCCXLIX = 1749）。</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>法国, 代用币, 里昂, 文学院, Jeton</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>¥268</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>268</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>竞宝斋</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>images/FJ-005.jpg</t>
+        </is>
+      </c>
+      <c r="V41" t="n">
+        <v>2882008</v>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>2026-07-12T16:22:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix FJ-005 card format: match FJ-004 new structure with coin-detail grid and description header
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:08</t>
+          <t>2026-07-12T16:30:53</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:53</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:53</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:53</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:09</t>
+          <t>2026-07-12T16:30:54</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4585,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr"/>
@@ -4814,7 +4814,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
     </row>
@@ -4937,6 +4937,46 @@
           <t>FJ-005</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ATHENAEUM LUGDUNENSE RESTITUTUM</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>法国 · 里昂文学院 银质代用币</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>ATHENAEUM LUGDUNENSE RESTITUTUM · Jeton en Argent · 1749</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>AD 1749 · 路易十五时期</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Jeton 银质代用币</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>银 · 30.2mm/9.28g</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr">
         <is>
           <t>FJ</t>
@@ -4944,17 +4984,17 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>法国王室纹章（蓝底三朵百合花）置于纹章框内，两侧为里昂守护神——持桨的罗讷河神（DVX）与持立标的索恩河神（SAO）。</t>
+          <t>正面: 法国王室纹章（蓝底三朵百合花）置于纹章框内，两侧为里昂守护神——持桨的罗讷河神（DVX）与持立标的索恩河神（SAO）。</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>柱廊神庙，上方两位胜利女神持桂冠；铭文「ATHENAEUM LUGDUNENSE RESTITUTUM」（里昂文学院重建），年铭「ACADEM. LITTER. LUGDUN. MDCCXLIX」（MDCCXLIX = 1749）。</t>
+          <t>反面: 柱廊神庙，上方两位胜利女神持桂冠；铭文「ATHENAEUM LUGDUNENSE RESTITUTUM」（里昂文学院重建），年铭「ACADEM. LITTER. LUGDUN. MDCCXLIX」（MDCCXLIX = 1749）。</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>法国, 代用币, 里昂, 文学院, Jeton</t>
+          <t>FJ, 法国, 代用币, jeton, 银, 1749, 里昂, 文学院, D.V., 学术, 胜利女神</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -4993,9 +5033,14 @@
       <c r="V41" t="n">
         <v>2882008</v>
       </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>此为 1749 年法国里昂文学院（Athenaeum Lugdunense）银质代用币（Jeton），雕刻师 D.V.（Dollin?）。里昂文学院成立于 1700 年，1749 年经历重建（Restitutum），此币为纪念重建而发行。&lt;br&gt;&lt;br&gt;&lt;strong&gt;关于 ATHENAEUM LUGDUNENSE&lt;/strong&gt;：里昂文学院是法国里昂市最重要的学术机构，由亨利四世于 1600 年设立，后于 1700 年正式确立。1749 年的「重建」（Restitutum）标志着该学院在经历了一段困难时期后的重新振兴。此 jeton 即为纪念这一学术复兴而铸。&lt;br&gt;&lt;br&gt;&lt;strong&gt;设计与象征&lt;/strong&gt;：正面为法国王室纹章（蓝底金鳖百合花），两侧分别持桨的罗讷河神（DVX）与持立标的索恩河神（SAO），象征里昂作为两河交汇之城的地理身份。背面为古典柱廊神庙，上方两位胜利女神（Victoria）持桂冠，象征学术与知识的胜利。&lt;br&gt;&lt;br&gt;&lt;strong&gt;铭文解读&lt;/strong&gt;：ATHENAEUM LUGDUNENSE RESTITUTUM = 里昂文学院重建；ACADEM. LITTER. LUGDUN. MDCCXLIX = MDCCXLIX = 1749 年。&lt;br&gt;&lt;br&gt;&lt;strong&gt;收藏价值&lt;/strong&gt;：里昂文学院 jeton 是法国学术史系列的重要代表，存世量有限。参考目录：Feuardent《Les Jetons français》、Ciani《Les Jetons français》。</t>
+        </is>
+      </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-07-12T16:22:10</t>
+          <t>2026-07-12T16:30:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix FJ-005: remove duplicate card stub, clean HTML structure
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:53</t>
+          <t>2026-07-12T16:47:54</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:53</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:53</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:53</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:54</t>
+          <t>2026-07-12T16:47:55</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4585,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr"/>
@@ -4814,7 +4814,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5040,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-07-12T16:30:55</t>
+          <t>2026-07-12T16:47:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-enter FJ-005 Lyon Athenaeum jeton 1749 with correct description; rebuild archive
</commit_message>
<xml_diff>
--- a/coin-archive/coins.xlsx
+++ b/coin-archive/coins.xlsx
@@ -690,7 +690,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:54</t>
+          <t>2026-07-12T16:58:25</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:25</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:25</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:25</t>
         </is>
       </c>
     </row>
@@ -1245,7 +1245,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:25</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2787,7 @@
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3568,7 @@
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:55</t>
+          <t>2026-07-12T16:58:26</t>
         </is>
       </c>
     </row>
@@ -3907,7 +3907,7 @@
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:27</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:27</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4133,7 @@
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:27</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:27</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="X35" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:27</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:27</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4585,7 @@
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:27</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="X38" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:27</t>
         </is>
       </c>
       <c r="Y38" t="inlineStr"/>
@@ -4814,7 +4814,7 @@
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:27</t>
         </is>
       </c>
     </row>
@@ -4927,7 +4927,7 @@
       </c>
       <c r="X40" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:27</t>
         </is>
       </c>
     </row>
@@ -4937,92 +4937,14 @@
           <t>FJ-005</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>ATHENAEUM LUGDUNENSE RESTITUTUM</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>法国 · 里昂文学院 银质代用币</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>ATHENAEUM LUGDUNENSE RESTITUTUM · Jeton en Argent · 1749</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>AD 1749 · 路易十五时期</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Jeton 银质代用币</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>银 · 30.2mm/9.28g</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="J41" t="inlineStr">
         <is>
           <t>FJ</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>正面: 法国王室纹章（蓝底三朵百合花）置于纹章框内，两侧为里昂守护神——持桨的罗讷河神（DVX）与持立标的索恩河神（SAO）。</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>反面: 柱廊神庙，上方两位胜利女神持桂冠；铭文「ATHENAEUM LUGDUNENSE RESTITUTUM」（里昂文学院重建），年铭「ACADEM. LITTER. LUGDUN. MDCCXLIX」（MDCCXLIX = 1749）。</t>
-        </is>
-      </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>FJ, 法国, 代用币, jeton, 银, 1749, 里昂, 文学院, D.V., 学术, 胜利女神</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>¥268</t>
-        </is>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>CNY</t>
-        </is>
-      </c>
-      <c r="P41" t="n">
-        <v>268</v>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>竞宝斋</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
-        <is>
-          <t>2024-08</t>
-        </is>
-      </c>
-      <c r="T41" t="inlineStr">
-        <is>
-          <t>2024</t>
+          <t>FJ, 法国, Jeton, 里昂, 1749</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -5035,12 +4957,12 @@
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>此为 1749 年法国里昂文学院（Athenaeum Lugdunense）银质代用币（Jeton），雕刻师 D.V.（Dollin?）。里昂文学院成立于 1700 年，1749 年经历重建（Restitutum），此币为纪念重建而发行。&lt;br&gt;&lt;br&gt;&lt;strong&gt;关于 ATHENAEUM LUGDUNENSE&lt;/strong&gt;：里昂文学院是法国里昂市最重要的学术机构，由亨利四世于 1600 年设立，后于 1700 年正式确立。1749 年的「重建」（Restitutum）标志着该学院在经历了一段困难时期后的重新振兴。此 jeton 即为纪念这一学术复兴而铸。&lt;br&gt;&lt;br&gt;&lt;strong&gt;设计与象征&lt;/strong&gt;：正面为法国王室纹章（蓝底金鳖百合花），两侧分别持桨的罗讷河神（DVX）与持立标的索恩河神（SAO），象征里昂作为两河交汇之城的地理身份。背面为古典柱廊神庙，上方两位胜利女神（Victoria）持桂冠，象征学术与知识的胜利。&lt;br&gt;&lt;br&gt;&lt;strong&gt;铭文解读&lt;/strong&gt;：ATHENAEUM LUGDUNENSE RESTITUTUM = 里昂文学院重建；ACADEM. LITTER. LUGDUN. MDCCXLIX = MDCCXLIX = 1749 年。&lt;br&gt;&lt;br&gt;&lt;strong&gt;收藏价值&lt;/strong&gt;：里昂文学院 jeton 是法国学术史系列的重要代表，存世量有限。参考目录：Feuardent《Les Jetons français》、Ciani《Les Jetons français》。</t>
+          <t>&lt;span class="obv-rev"&gt;📜 历史背景&lt;/span&gt;</t>
         </is>
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>2026-07-12T16:47:56</t>
+          <t>2026-07-12T16:58:27</t>
         </is>
       </c>
     </row>

</xml_diff>